<commit_message>
Drop ARI:0001168 from the reports and regenerate downstream outputs
Remove Primary immune deficiency from 1_Core_ARI_Diseases.xlsx and
4_Additional_Info_Index.xlsx, shifting hyperlinks with their rows, then
rerun the grounding pipeline and the disease-target matrix. The grounding
CSVs lose only that row. Reports 6 and 8 also catch up with changes made
since they were last generated: the ICD-9 xref grouping and the current
mapping set, which replaces the stale ARI:0003 rows.

The four older grounding scripts pointed at a /sessions sandbox path;
they now resolve repo files relative to the script so they can run here.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/4-reports/1_Core_ARI_Diseases.xlsx
+++ b/data/4-reports/1_Core_ARI_Diseases.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core ARI Diseases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Core ARI Diseases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Core ARI Diseases'!$A$1:$P$1</definedName>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P212"/>
+  <dimension ref="A1:P211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -11141,117 +11141,133 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001168</t>
+          <t>ARI:0001169</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001168</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001169</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>Primary immune deficiency</t>
-        </is>
-      </c>
-      <c r="D169" s="4" t="inlineStr"/>
-      <c r="E169" s="4" t="inlineStr">
-        <is>
-          <t>STAT3 gain-of-function disease; Combined immunodeficiency disease; Autosomal recessive SCID (severe combined immunodeficiency disease); Congenital immunodeficiency disease; Severe combined immunodeficiency disease; Hypopigmentation-immunodeficiency disease</t>
-        </is>
-      </c>
+          <t>Primary sclerosing cholangitis</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>Chronic obliterative cholangitis; Fibrosing cholangitis; PSC; Stenosing cholangitis</t>
+        </is>
+      </c>
+      <c r="E169" s="4" t="inlineStr"/>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>442459007, 362993009, 36138009, 31323000, 37548006</t>
+          <t>197441003</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr"/>
       <c r="H169" s="3" t="inlineStr">
         <is>
-          <t>40483560, 4179989, 4263109, 29783, 4292707</t>
-        </is>
-      </c>
-      <c r="I169" s="2" t="inlineStr"/>
+          <t>4058821</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>197441003</t>
+        </is>
+      </c>
       <c r="J169" s="2" t="inlineStr"/>
-      <c r="K169" s="4" t="inlineStr"/>
-      <c r="L169" s="4" t="inlineStr"/>
+      <c r="K169" s="4" t="inlineStr">
+        <is>
+          <t>PSC is a rare progressive disorder of the liver which is characterized by inflammation, thickening, and abnormal formation of fibrous tissue within the passages that carry bile from the liver (bile ducts). Both bile ducts within the liver and outside the liver are affected.</t>
+        </is>
+      </c>
+      <c r="L169" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liang 2017; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC5478316/ </t>
+        </is>
+      </c>
       <c r="M169" s="2" t="inlineStr">
         <is>
-          <t>Immune System</t>
-        </is>
-      </c>
-      <c r="N169" s="2" t="inlineStr"/>
+          <t>Liver</t>
+        </is>
+      </c>
+      <c r="N169" s="2" t="inlineStr">
+        <is>
+          <t>TCELL</t>
+        </is>
+      </c>
       <c r="O169" s="2" t="inlineStr">
         <is>
-          <t>Dysregulation</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P169" s="2" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001169</t>
+          <t>ARI:0001170</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001169</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001170</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>Primary sclerosing cholangitis</t>
+          <t>Progressive hemifacial atrophy</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>Chronic obliterative cholangitis; Fibrosing cholangitis; PSC; Stenosing cholangitis</t>
+          <t>Idiopathic hemifacial atrophy; Parry Romberg syndrome; Progressive facial hemiatrophy; Romberg's syndrome</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr"/>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>197441003</t>
+          <t>718224004</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr"/>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>4058821</t>
+          <t>37397558</t>
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>197441003</t>
+          <t>718224004</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr"/>
       <c r="K170" s="4" t="inlineStr">
         <is>
-          <t>PSC is a rare progressive disorder of the liver which is characterized by inflammation, thickening, and abnormal formation of fibrous tissue within the passages that carry bile from the liver (bile ducts). Both bile ducts within the liver and outside the liver are affected.</t>
+          <t xml:space="preserve">Progressive hemifacial atrophy, also called Parry Romberg Syndrome, predominantly affects the skin of the face and is believed to be autoimmune in nature, though the cause is still being researched.  Typically, the skin deteriorates gradually over one side of the face, beginning with the upper jaw and the area extending from the nose to the corner of the lip, and then spreading to other parts of the face.  In some cases, symptoms are not restricted to only one side of the face and may also occur in the trunk or limbs.  Severe cases can spread to the muscles, bones, and cartilage.  Patients can expect symptoms to progress over a period of 2 to 20 years, after which time progression plateaus.  Treatments have so far been unsuccessful in stopping progression, but they do help manage associated discomfort.  Cases that progress over longer periods of time and beginning at a younger age often lead to the most severe symptoms, resulting in facial distortions and nerve disorders. </t>
         </is>
       </c>
       <c r="L170" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liang 2017; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC5478316/ </t>
+          <t>Gupta 2016; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4991159/</t>
         </is>
       </c>
       <c r="M170" s="2" t="inlineStr">
         <is>
-          <t>Liver</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="N170" s="2" t="inlineStr">
         <is>
-          <t>TCELL</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="O170" s="2" t="inlineStr">
         <is>
-          <t>Autoimmune</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="P170" s="2" t="n">
@@ -11261,130 +11277,134 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001170</t>
+          <t>ARI:0001171</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001170</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001171</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Progressive hemifacial atrophy</t>
-        </is>
-      </c>
-      <c r="D171" s="4" t="inlineStr">
-        <is>
-          <t>Idiopathic hemifacial atrophy; Parry Romberg syndrome; Progressive facial hemiatrophy; Romberg's syndrome</t>
-        </is>
-      </c>
-      <c r="E171" s="4" t="inlineStr"/>
+          <t>Psoriasis</t>
+        </is>
+      </c>
+      <c r="D171" s="4" t="inlineStr"/>
+      <c r="E171" s="4" t="inlineStr">
+        <is>
+          <t>Guttate psoriasis</t>
+        </is>
+      </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>718224004</t>
+          <t>37042000, 9014002</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr"/>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>37397558</t>
+          <t>4284492, 140168</t>
         </is>
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>718224004</t>
+          <t>37042000, 9014002</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr"/>
       <c r="K171" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Progressive hemifacial atrophy, also called Parry Romberg Syndrome, predominantly affects the skin of the face and is believed to be autoimmune in nature, though the cause is still being researched.  Typically, the skin deteriorates gradually over one side of the face, beginning with the upper jaw and the area extending from the nose to the corner of the lip, and then spreading to other parts of the face.  In some cases, symptoms are not restricted to only one side of the face and may also occur in the trunk or limbs.  Severe cases can spread to the muscles, bones, and cartilage.  Patients can expect symptoms to progress over a period of 2 to 20 years, after which time progression plateaus.  Treatments have so far been unsuccessful in stopping progression, but they do help manage associated discomfort.  Cases that progress over longer periods of time and beginning at a younger age often lead to the most severe symptoms, resulting in facial distortions and nerve disorders. </t>
-        </is>
-      </c>
-      <c r="L171" s="4" t="inlineStr">
-        <is>
-          <t>Gupta 2016; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4991159/</t>
-        </is>
-      </c>
-      <c r="M171" s="2" t="inlineStr">
-        <is>
-          <t>Skin</t>
-        </is>
-      </c>
-      <c r="N171" s="2" t="inlineStr">
-        <is>
-          <t>Unconfirmed</t>
-        </is>
-      </c>
-      <c r="O171" s="2" t="inlineStr">
-        <is>
-          <t>Unconfirmed</t>
-        </is>
-      </c>
-      <c r="P171" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001171</t>
-        </is>
-      </c>
-      <c r="B172" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001171</t>
-        </is>
-      </c>
-      <c r="C172" s="2" t="inlineStr">
-        <is>
-          <t>Psoriasis</t>
-        </is>
-      </c>
-      <c r="D172" s="4" t="inlineStr"/>
-      <c r="E172" s="4" t="inlineStr">
-        <is>
-          <t>Guttate psoriasis</t>
-        </is>
-      </c>
-      <c r="F172" s="3" t="inlineStr">
-        <is>
-          <t>37042000, 9014002</t>
-        </is>
-      </c>
-      <c r="G172" s="2" t="inlineStr"/>
-      <c r="H172" s="3" t="inlineStr">
-        <is>
-          <t>4284492, 140168</t>
-        </is>
-      </c>
-      <c r="I172" s="2" t="inlineStr">
-        <is>
-          <t>37042000, 9014002</t>
-        </is>
-      </c>
-      <c r="J172" s="2" t="inlineStr"/>
-      <c r="K172" s="4" t="inlineStr">
         <is>
           <t>Psoriasis is a chronic autoimmune disease that causes raised, red, scaly patches to appear on the skin. It affects 1% to 3% of people in Western countries. Psoriasis can appear anywhere on the body, with some cases being mild and others severe enough to significantly impact quality of life. The condition can develop at any age, with earlier onset associated with more severe disease than later onset. Various triggers, including trauma, infections, dry skin, and certain medications, can worsen the condition. Some people with psoriasis may also develop psoriatic arthritis, which causes joint pain and stiffness.
 The disease is caused by an overactive immune system, where T cells mistakenly attack the skin, leading to inflammation and rapid skin cell turnover. This process is driven by immune system proteins called cytokines, such as IL-23 and TNF-α, which promote inflammation. Treatments targeting these immune responses, such as biologic medications and immunosuppressants, have been effective in managing symptoms. Despite its autoimmune features, researchers have yet to identify the exact self-antigen that triggers the immune response in psoriasis.
 The development of psoriasis involves a complex cycle of immune activation and skin cell dysfunction. Triggers such as physical injury or infections can initiate an immune response that leads to inflammation and the recruitment of immune cells into the skin. These immune cells release cytokines that further stimulate skin cells, causing thickening and scaling. While genetic factors play a role in susceptibility, environmental triggers are also important. Ongoing research aims to better understand the disease mechanisms and develop more targeted therapies to improve treatment outcomes.</t>
         </is>
       </c>
+      <c r="L171" s="4" t="inlineStr">
+        <is>
+          <t>Rachakonda 2014; https://pubmed.ncbi.nlm.nih.gov/24388724/</t>
+        </is>
+      </c>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>Skin</t>
+        </is>
+      </c>
+      <c r="N171" s="2" t="inlineStr">
+        <is>
+          <t>TCELL</t>
+        </is>
+      </c>
+      <c r="O171" s="2" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="P171" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001172</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001172</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Psoriatic arthritis</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>PsA</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="inlineStr"/>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>156370009, 33339001</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>33339001</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>81931, 40319772</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>156370009, 33339001</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr"/>
+      <c r="K172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Psoriatic arthritis is an autoimmune disease marked by the combination of psoriasis and one or more forms of rheumatoid-like arthritis, including anklosing spondylitis, rheumatoid arthritis, and juvenile rheumatoid arthritis. </t>
+        </is>
+      </c>
       <c r="L172" s="4" t="inlineStr">
         <is>
-          <t>Rachakonda 2014; https://pubmed.ncbi.nlm.nih.gov/24388724/</t>
+          <t>Ogdie 2015; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4610151/pdf/nihms-710337.pdf</t>
         </is>
       </c>
       <c r="M172" s="2" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>Musculoskeletal</t>
         </is>
       </c>
       <c r="N172" s="2" t="inlineStr">
         <is>
-          <t>TCELL</t>
+          <t>Immune-mediated</t>
         </is>
       </c>
       <c r="O172" s="2" t="inlineStr">
@@ -11399,115 +11419,43 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001172</t>
+          <t>ARI:0001173</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001172</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001173</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>Psoriatic arthritis</t>
+          <t>Pure red cell aplasia</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>PsA</t>
+          <t xml:space="preserve">Acquired pure red cell aplasia; Adult pure red cell aplasia; Idiopathic pure red cell aplasia; PRCA; Primary acquired PRCA; Primary acquired pure red cell aplasia </t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr"/>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>156370009, 33339001</t>
-        </is>
-      </c>
-      <c r="G173" s="2" t="inlineStr">
-        <is>
-          <t>33339001</t>
-        </is>
-      </c>
+          <t>50715003</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr"/>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>81931, 40319772</t>
+          <t>140065</t>
         </is>
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>156370009, 33339001</t>
+          <t>50715003</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr"/>
       <c r="K173" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Psoriatic arthritis is an autoimmune disease marked by the combination of psoriasis and one or more forms of rheumatoid-like arthritis, including anklosing spondylitis, rheumatoid arthritis, and juvenile rheumatoid arthritis. </t>
-        </is>
-      </c>
-      <c r="L173" s="4" t="inlineStr">
-        <is>
-          <t>Ogdie 2015; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4610151/pdf/nihms-710337.pdf</t>
-        </is>
-      </c>
-      <c r="M173" s="2" t="inlineStr">
-        <is>
-          <t>Musculoskeletal</t>
-        </is>
-      </c>
-      <c r="N173" s="2" t="inlineStr">
-        <is>
-          <t>Immune-mediated</t>
-        </is>
-      </c>
-      <c r="O173" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
-      <c r="P173" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001173</t>
-        </is>
-      </c>
-      <c r="B174" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001173</t>
-        </is>
-      </c>
-      <c r="C174" s="2" t="inlineStr">
-        <is>
-          <t>Pure red cell aplasia</t>
-        </is>
-      </c>
-      <c r="D174" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Acquired pure red cell aplasia; Adult pure red cell aplasia; Idiopathic pure red cell aplasia; PRCA; Primary acquired PRCA; Primary acquired pure red cell aplasia </t>
-        </is>
-      </c>
-      <c r="E174" s="4" t="inlineStr"/>
-      <c r="F174" s="3" t="inlineStr">
-        <is>
-          <t>50715003</t>
-        </is>
-      </c>
-      <c r="G174" s="2" t="inlineStr"/>
-      <c r="H174" s="3" t="inlineStr">
-        <is>
-          <t>140065</t>
-        </is>
-      </c>
-      <c r="I174" s="2" t="inlineStr">
-        <is>
-          <t>50715003</t>
-        </is>
-      </c>
-      <c r="J174" s="2" t="inlineStr"/>
-      <c r="K174" s="4" t="inlineStr">
         <is>
           <t>Pure red cell aplasia (PRCA) occurs when red blood cells fail to fully develop after they are produced in the bone marrow.  This leads to symptoms of anemia, including tiredness and pale skin.  There are 2 types of PRCA caused by autoimmune processes:  
 Acquired primary PRCA typically affects adults and leads to symptoms of anemia.  The trigger for primary PRCA is unknown. Acquired primary PRCA is caused by the immune system attacking developing red blood cells, preventing them from maturing into functional adult cells.  
@@ -11516,24 +11464,89 @@
 A third type of PRCA, Diamond-Blackfan syndrome, is due to genetic mutation and presents during infancy.   It is not autoimmune.</t>
         </is>
       </c>
+      <c r="L173" s="4" t="inlineStr">
+        <is>
+          <t>Nakazawa 2022; https://pubmed.ncbi.nlm.nih.gov/35522950/</t>
+        </is>
+      </c>
+      <c r="M173" s="2" t="inlineStr">
+        <is>
+          <t>Blood</t>
+        </is>
+      </c>
+      <c r="N173" s="2" t="inlineStr">
+        <is>
+          <t>Antibody</t>
+        </is>
+      </c>
+      <c r="O173" s="2" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="P173" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001174</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001174</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Pyoderma gangrenosum</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr"/>
+      <c r="E174" s="4" t="inlineStr"/>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>74578003</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr"/>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>133283</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>74578003</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr"/>
+      <c r="K174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pyoderma gangrenosum is an autoinflammatory skin disease that starts as small red bumps and develops into large open sores on the skin, usually on the legs.
+</t>
+        </is>
+      </c>
       <c r="L174" s="4" t="inlineStr">
         <is>
-          <t>Nakazawa 2022; https://pubmed.ncbi.nlm.nih.gov/35522950/</t>
+          <t>Xu 2020; https://pubmed.ncbi.nlm.nih.gov/31400451/</t>
         </is>
       </c>
       <c r="M174" s="2" t="inlineStr">
         <is>
-          <t>Blood</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="N174" s="2" t="inlineStr">
         <is>
-          <t>Antibody</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="O174" s="2" t="inlineStr">
         <is>
-          <t>Autoimmune</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="P174" s="2" t="n">
@@ -11543,62 +11556,61 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001174</t>
+          <t>ARI:0001175</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001174</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001175</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>Pyoderma gangrenosum</t>
+          <t>Rasmussen syndrome</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr"/>
       <c r="E175" s="4" t="inlineStr"/>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>74578003</t>
+          <t>230191005, 435341000124104</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr"/>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>133283</t>
+          <t>4041672, 763040</t>
         </is>
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>74578003</t>
+          <t>230191005, 435341000124104</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr"/>
       <c r="K175" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pyoderma gangrenosum is an autoinflammatory skin disease that starts as small red bumps and develops into large open sores on the skin, usually on the legs.
-</t>
+          <t>Rasmussen syndrome, or Rasmussen’s Encephalitis (RE), is a rare, progressive disease that involves cognitive decline due to inflammation of one half of the brain. Those with Rasmussen syndrome experience frequent seizures and eventual permanent brain damage. This disease mostly affects children ages 2 and 10, but can also affect adolescents and adults. Treatments for this disease include antiseizure medication, immunotherapy, and in more severe cases, brain surgery. The cause of Rasmussen's syndrome is unknown, however, researchers believe that it may be an autoimmune condition that affects one half of the brain or may occur due to an unknown virus entering the brain.</t>
         </is>
       </c>
       <c r="L175" s="4" t="inlineStr">
         <is>
-          <t>Xu 2020; https://pubmed.ncbi.nlm.nih.gov/31400451/</t>
+          <t>Bien 2013; https://pubmed.ncbi.nlm.nih.gov/23216622/</t>
         </is>
       </c>
       <c r="M175" s="2" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>Nervous System</t>
         </is>
       </c>
       <c r="N175" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Antibody</t>
         </is>
       </c>
       <c r="O175" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P175" s="2" t="n">
@@ -11608,61 +11620,66 @@
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001175</t>
+          <t>ARI:0001176</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001175</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001176</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>Rasmussen syndrome</t>
-        </is>
-      </c>
-      <c r="D176" s="4" t="inlineStr"/>
+          <t>Secondary Raynaud's phenomenon</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>Raynaud disease; Raynaud's disease; Raynaud's phenomenon; Secondary Raynaud's</t>
+        </is>
+      </c>
       <c r="E176" s="4" t="inlineStr"/>
       <c r="F176" s="3" t="inlineStr">
         <is>
-          <t>230191005, 435341000124104</t>
+          <t>356198000, 266261006</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr"/>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>4041672, 763040</t>
+          <t>4143972, 4229162</t>
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>230191005, 435341000124104</t>
+          <t>356198000, 266261006</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr"/>
       <c r="K176" s="4" t="inlineStr">
         <is>
-          <t>Rasmussen syndrome, or Rasmussen’s Encephalitis (RE), is a rare, progressive disease that involves cognitive decline due to inflammation of one half of the brain. Those with Rasmussen syndrome experience frequent seizures and eventual permanent brain damage. This disease mostly affects children ages 2 and 10, but can also affect adolescents and adults. Treatments for this disease include antiseizure medication, immunotherapy, and in more severe cases, brain surgery. The cause of Rasmussen's syndrome is unknown, however, researchers believe that it may be an autoimmune condition that affects one half of the brain or may occur due to an unknown virus entering the brain.</t>
+          <t>In secondary Raynaud's phenomenon, blood flow to the fingers and toes is limited, causing cold extremities and sometimes pain. The condition is made worse by cold temperatures. The amount of time that these extremities stay cold can vary.  
+Secondary Raynaud's is a symptom experienced (and reported) by patients with autoimmune diseases.  Primary Raynaud's is when the symptoms appear without any other disease.  Therefore, primary Raynaud's is not an autoimmune disease.  However, a person suffering from Raynaud's could have an undiagnosed autoimmune disease.</t>
         </is>
       </c>
       <c r="L176" s="4" t="inlineStr">
         <is>
-          <t>Bien 2013; https://pubmed.ncbi.nlm.nih.gov/23216622/</t>
+          <t>Garner 2015; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4368987/</t>
         </is>
       </c>
       <c r="M176" s="2" t="inlineStr">
         <is>
-          <t>Nervous System</t>
+          <t>Vascular system</t>
         </is>
       </c>
       <c r="N176" s="2" t="inlineStr">
         <is>
-          <t>Antibody</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="O176" s="2" t="inlineStr">
         <is>
-          <t>Autoimmune</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="P176" s="2" t="n">
@@ -11672,66 +11689,65 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001176</t>
+          <t>ARI:0001177</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001176</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001177</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>Secondary Raynaud's phenomenon</t>
+          <t>Reactive arthritis</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>Raynaud disease; Raynaud's disease; Raynaud's phenomenon; Secondary Raynaud's</t>
+          <t>Fiessinger-Leroy disease; ReA; Reactive arthritis triad; Reiter's syndrome</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr"/>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>356198000, 266261006</t>
+          <t>201736002, 67224007</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr"/>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>4143972, 4229162</t>
+          <t>40399768, 78357</t>
         </is>
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>356198000, 266261006</t>
+          <t>201736002, 67224007</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr"/>
       <c r="K177" s="4" t="inlineStr">
         <is>
-          <t>In secondary Raynaud's phenomenon, blood flow to the fingers and toes is limited, causing cold extremities and sometimes pain. The condition is made worse by cold temperatures. The amount of time that these extremities stay cold can vary.  
-Secondary Raynaud's is a symptom experienced (and reported) by patients with autoimmune diseases.  Primary Raynaud's is when the symptoms appear without any other disease.  Therefore, primary Raynaud's is not an autoimmune disease.  However, a person suffering from Raynaud's could have an undiagnosed autoimmune disease.</t>
+          <t xml:space="preserve">Reactive arthritis is an autoimmune condition classified in the family of spondyloarthritis. It is a type of arthritis that is typically acute and is most frequently caused by infections from bacteria in the genitals or bowel.  Reactive arthritis symptoms usually last for between 3 and 12 months. However, in some individuals, subsequent flares may occur due to stress or infection. The condition may also become chronic in some individuals.  Reactive arthritis may go unnoticed and heal on its own or it can cause pain in the joints. The knees and ankles are affected most often. </t>
         </is>
       </c>
       <c r="L177" s="4" t="inlineStr">
         <is>
-          <t>Garner 2015; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4368987/</t>
+          <t>Hanova 2010; https://pubmed.ncbi.nlm.nih.gov/20476864/</t>
         </is>
       </c>
       <c r="M177" s="2" t="inlineStr">
         <is>
-          <t>Vascular system</t>
+          <t>Musculoskeletal</t>
         </is>
       </c>
       <c r="N177" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Immune-mediated</t>
         </is>
       </c>
       <c r="O177" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P177" s="2" t="n">
@@ -11741,50 +11757,51 @@
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001177</t>
+          <t>ARI:0001178</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001177</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001178</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Reactive arthritis</t>
+          <t>Relapsing polychondritis</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>Fiessinger-Leroy disease; ReA; Reactive arthritis triad; Reiter's syndrome</t>
+          <t>Atrophic polychondritis; Chronic atrophic polychondritis; Meyenburg-Altherr-Uehlinger syndrome; Polychondropathia; Recurrent polychondritis; Relapsing perichondritis; Relapsing polyneuropathy; Systemic chondromalacia; Systemic chondromalocia; Von Meyenburg disease</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr"/>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>201736002, 67224007</t>
+          <t>72275000</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr"/>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>40399768, 78357</t>
+          <t>4216873</t>
         </is>
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>201736002, 67224007</t>
+          <t>72275000, 72275001</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr"/>
       <c r="K178" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reactive arthritis is an autoimmune condition classified in the family of spondyloarthritis. It is a type of arthritis that is typically acute and is most frequently caused by infections from bacteria in the genitals or bowel.  Reactive arthritis symptoms usually last for between 3 and 12 months. However, in some individuals, subsequent flares may occur due to stress or infection. The condition may also become chronic in some individuals.  Reactive arthritis may go unnoticed and heal on its own or it can cause pain in the joints. The knees and ankles are affected most often. </t>
+          <t xml:space="preserve">Relapsing polychondritis (RP) occurs when the immune system attacks cartilage and other related tissues in the body, causing inflammation and tissue damage. Though the disease is frequently characterized through ears, nose, and joint symptoms, it is a multi-systemic disease. Episodes may last several days to weeks and typically resolve without treatment. 
+In cases where the cartilage is not visible, RP can cause heart valve abnormalities, kidney disease, neurological problems, gastrointestinal problems.  </t>
         </is>
       </c>
       <c r="L178" s="4" t="inlineStr">
         <is>
-          <t>Hanova 2010; https://pubmed.ncbi.nlm.nih.gov/20476864/</t>
+          <t>Kent 2004; https://pubmed.ncbi.nlm.nih.gov/14673390/</t>
         </is>
       </c>
       <c r="M178" s="2" t="inlineStr">
@@ -11794,7 +11811,7 @@
       </c>
       <c r="N178" s="2" t="inlineStr">
         <is>
-          <t>Immune-mediated</t>
+          <t>Antibody</t>
         </is>
       </c>
       <c r="O178" s="2" t="inlineStr">
@@ -11809,66 +11826,65 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001178</t>
+          <t>ARI:0001179</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001178</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001179</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Relapsing polychondritis</t>
+          <t>Restless legs</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>Atrophic polychondritis; Chronic atrophic polychondritis; Meyenburg-Altherr-Uehlinger syndrome; Polychondropathia; Recurrent polychondritis; Relapsing perichondritis; Relapsing polyneuropathy; Systemic chondromalacia; Systemic chondromalocia; Von Meyenburg disease</t>
+          <t>Restless leg syndrome; Willis-Ekbom Disease</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr"/>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>72275000</t>
+          <t>32914008</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr"/>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>4216873</t>
+          <t>73754</t>
         </is>
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>72275000, 72275001</t>
+          <t>32914008</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr"/>
       <c r="K179" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relapsing polychondritis (RP) occurs when the immune system attacks cartilage and other related tissues in the body, causing inflammation and tissue damage. Though the disease is frequently characterized through ears, nose, and joint symptoms, it is a multi-systemic disease. Episodes may last several days to weeks and typically resolve without treatment. 
-In cases where the cartilage is not visible, RP can cause heart valve abnormalities, kidney disease, neurological problems, gastrointestinal problems.  </t>
+          <t>A condition that causes an unpleasant or uncomfortable sensation in the legs and an irresistible urge to move them.  Restless leg syndrome is a symptom of several autoimmune diseases, including &lt;a href="/Disease_Profile/rheumatoid-arthritis.aspx"&gt;rheumatoid arthritis, &lt;a href="/Disease_Profile/Sj%C3%B6grens-disease.aspx"&gt;Sjögren's disease, &lt;a href="/Disease_Profile/crohns-disease.aspx"&gt;Crohn's disease&lt;/a&gt;, and other inflammatory bowel diseases.  However, since restless leg is a relatively common condition affecting 8% of the population, the correlation with autoimmune disease might not indicate a causative relationship.</t>
         </is>
       </c>
       <c r="L179" s="4" t="inlineStr">
         <is>
-          <t>Kent 2004; https://pubmed.ncbi.nlm.nih.gov/14673390/</t>
+          <t xml:space="preserve"> Innes 2011 ; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4634567/</t>
         </is>
       </c>
       <c r="M179" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal</t>
+          <t>Nervous System</t>
         </is>
       </c>
       <c r="N179" s="2" t="inlineStr">
         <is>
-          <t>Antibody</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="O179" s="2" t="inlineStr">
         <is>
-          <t>Autoimmune</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="P179" s="2" t="n">
@@ -11878,65 +11894,66 @@
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001179</t>
+          <t>ARI:0001180</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001179</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001180</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Restless legs</t>
+          <t>Retinocochleocerebral vasculopathy</t>
         </is>
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>Restless leg syndrome; Willis-Ekbom Disease</t>
+          <t>RED-M; Retinopathy-encephalopathy-deafness associated microangiopathy; SICRET; Small infarctions of cochlear, retinal and encephalic tissue; Susac syndrome; Susac's syndrome</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr"/>
       <c r="F180" s="3" t="inlineStr">
         <is>
-          <t>32914008</t>
+          <t>702575003</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr"/>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>73754</t>
+          <t>45765600</t>
         </is>
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>32914008</t>
+          <t>702575003</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr"/>
       <c r="K180" s="4" t="inlineStr">
         <is>
-          <t>A condition that causes an unpleasant or uncomfortable sensation in the legs and an irresistible urge to move them.  Restless leg syndrome is a symptom of several autoimmune diseases, including &lt;a href="/Disease_Profile/rheumatoid-arthritis.aspx"&gt;rheumatoid arthritis, &lt;a href="/Disease_Profile/Sj%C3%B6grens-disease.aspx"&gt;Sjögren's disease, &lt;a href="/Disease_Profile/crohns-disease.aspx"&gt;Crohn's disease&lt;/a&gt;, and other inflammatory bowel diseases.  However, since restless leg is a relatively common condition affecting 8% of the population, the correlation with autoimmune disease might not indicate a causative relationship.</t>
+          <t>Susac's syndrome affects three parts of the body: the brain, the retina of the eye, and the inner ear. The cause is uncertain, but the disease is believed to be autoimmune.  Swelling in the lining of the blood vessels in these three areas blocks and decreases blood flow, which results in impaired brain function and vision/ hearing loss.  Symptoms are typically unstable as the disease progresses, and patients often experience disturbance in only 2 of the 3 areas at any given time.  
+The severity of cases may vary, with mild cases resolving in under a year and severe cases having longer duration and causing irreparable damage.  During the course of the disease, some patients may experience symptoms in a flare-remission pattern, while others are consistently symptomatic until time of recovery.  Treatment is available to prevent permanent damage, and most patients under medical care can expect to experience complete or near complete recovery.</t>
         </is>
       </c>
       <c r="L180" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Innes 2011 ; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4634567/</t>
+          <t>Dörr 2013; https://pubmed.ncbi.nlm.nih.gov/23628737/</t>
         </is>
       </c>
       <c r="M180" s="2" t="inlineStr">
         <is>
-          <t>Nervous System</t>
+          <t>Vascular system</t>
         </is>
       </c>
       <c r="N180" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Antibody Suspected</t>
         </is>
       </c>
       <c r="O180" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P180" s="2" t="n">
@@ -11946,66 +11963,66 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001180</t>
+          <t>ARI:0001181</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001180</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001181</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Retinocochleocerebral vasculopathy</t>
+          <t>Rheumatic Chorea</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>RED-M; Retinopathy-encephalopathy-deafness associated microangiopathy; SICRET; Small infarctions of cochlear, retinal and encephalic tissue; Susac syndrome; Susac's syndrome</t>
+          <t>St. Vitus Dance; Sydenham chorea; Syndenham chorea</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr"/>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>702575003</t>
+          <t>46826000</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr"/>
       <c r="H181" s="3" t="inlineStr">
         <is>
-          <t>45765600</t>
+          <t>444120</t>
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>702575003</t>
+          <t>46826000</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr"/>
       <c r="K181" s="4" t="inlineStr">
         <is>
-          <t>Susac's syndrome affects three parts of the body: the brain, the retina of the eye, and the inner ear. The cause is uncertain, but the disease is believed to be autoimmune.  Swelling in the lining of the blood vessels in these three areas blocks and decreases blood flow, which results in impaired brain function and vision/ hearing loss.  Symptoms are typically unstable as the disease progresses, and patients often experience disturbance in only 2 of the 3 areas at any given time.  
-The severity of cases may vary, with mild cases resolving in under a year and severe cases having longer duration and causing irreparable damage.  During the course of the disease, some patients may experience symptoms in a flare-remission pattern, while others are consistently symptomatic until time of recovery.  Treatment is available to prevent permanent damage, and most patients under medical care can expect to experience complete or near complete recovery.</t>
+          <t>Rheumatic chorea, also called Sydenham chorea, is a rare neurological disorder typically occurring during childhood. It is caused by an autoimmune reaction following infection from the same bacterium that causes rheumatic fever. It leads to chorea: sudden, continuous, involuntary movements affecting the entire body. Symptoms can last in children anywhere from 3 weeks to several months. Patients with mild cases recover on their own in a few weeks, but treatment is available to provide relief to those with severe symptoms.
+Since antibiotics have reduced the incidence of rheumatic fever, the incidence of rheumatic chorea in developed countries like the US is much lower than in developing countries. (Note that we could not find a study that supports a statistic cited in several papers that 30% of patients with rheumatic fever develop rheumatic chorea).</t>
         </is>
       </c>
       <c r="L181" s="4" t="inlineStr">
         <is>
-          <t>Dörr 2013; https://pubmed.ncbi.nlm.nih.gov/23628737/</t>
+          <t>No studies found; CONFIRMED NO DATA Sept 2021</t>
         </is>
       </c>
       <c r="M181" s="2" t="inlineStr">
         <is>
-          <t>Vascular system</t>
+          <t>Musculoskeletal</t>
         </is>
       </c>
       <c r="N181" s="2" t="inlineStr">
         <is>
-          <t>Antibody Suspected</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="O181" s="2" t="inlineStr">
         <is>
-          <t>Autoimmune</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="P181" s="2" t="n">
@@ -12015,112 +12032,43 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001181</t>
+          <t>ARI:0001182</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001181</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001182</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Rheumatic Chorea</t>
+          <t>Rheumatic fever</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>St. Vitus Dance; Sydenham chorea; Syndenham chorea</t>
+          <t>Acute rheumatic fever; Acute rheumatic myocarditis; Inflammatory rheumatism; Rheumatic arthritis</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr"/>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>46826000</t>
+          <t>58718002, 194709000</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr"/>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>444120</t>
+          <t>442313</t>
         </is>
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>46826000</t>
+          <t>58718002, 194709000</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr"/>
       <c r="K182" s="4" t="inlineStr">
-        <is>
-          <t>Rheumatic chorea, also called Sydenham chorea, is a rare neurological disorder typically occurring during childhood. It is caused by an autoimmune reaction following infection from the same bacterium that causes rheumatic fever. It leads to chorea: sudden, continuous, involuntary movements affecting the entire body. Symptoms can last in children anywhere from 3 weeks to several months. Patients with mild cases recover on their own in a few weeks, but treatment is available to provide relief to those with severe symptoms.
-Since antibiotics have reduced the incidence of rheumatic fever, the incidence of rheumatic chorea in developed countries like the US is much lower than in developing countries. (Note that we could not find a study that supports a statistic cited in several papers that 30% of patients with rheumatic fever develop rheumatic chorea).</t>
-        </is>
-      </c>
-      <c r="L182" s="4" t="inlineStr">
-        <is>
-          <t>No studies found; CONFIRMED NO DATA Sept 2021</t>
-        </is>
-      </c>
-      <c r="M182" s="2" t="inlineStr">
-        <is>
-          <t>Musculoskeletal</t>
-        </is>
-      </c>
-      <c r="N182" s="2" t="inlineStr">
-        <is>
-          <t>Unconfirmed</t>
-        </is>
-      </c>
-      <c r="O182" s="2" t="inlineStr">
-        <is>
-          <t>Unconfirmed</t>
-        </is>
-      </c>
-      <c r="P182" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001182</t>
-        </is>
-      </c>
-      <c r="B183" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001182</t>
-        </is>
-      </c>
-      <c r="C183" s="2" t="inlineStr">
-        <is>
-          <t>Rheumatic fever</t>
-        </is>
-      </c>
-      <c r="D183" s="4" t="inlineStr">
-        <is>
-          <t>Acute rheumatic fever; Acute rheumatic myocarditis; Inflammatory rheumatism; Rheumatic arthritis</t>
-        </is>
-      </c>
-      <c r="E183" s="4" t="inlineStr"/>
-      <c r="F183" s="3" t="inlineStr">
-        <is>
-          <t>58718002, 194709000</t>
-        </is>
-      </c>
-      <c r="G183" s="2" t="inlineStr"/>
-      <c r="H183" s="3" t="inlineStr">
-        <is>
-          <t>442313</t>
-        </is>
-      </c>
-      <c r="I183" s="2" t="inlineStr">
-        <is>
-          <t>58718002, 194709000</t>
-        </is>
-      </c>
-      <c r="J183" s="2" t="inlineStr"/>
-      <c r="K183" s="4" t="inlineStr">
         <is>
           <t>Rheumatic fever is an inflammatory disease that sometimes develops as a complication of inadequately treated strep throat (group A streptococcal infection). Rheumatic fever can cause permanent damage to the heart including damaged heart valves and heart failure.  The disease is mostly diagnosed in children.
 Rheumatic fever is not a chronic condition, but the consequences of the heart damage it may cause, rheumatic heart disease, can be chronic. 
@@ -12128,114 +12076,114 @@
 Note: scarlet fever is another symptom of a strep infection but is not a separate cause of rheumatic fever.</t>
         </is>
       </c>
-      <c r="L183" s="4" t="inlineStr">
+      <c r="L182" s="4" t="inlineStr">
         <is>
           <t>Orphanet; https://www.orpha.net/consor/cgi-bin/OC_Exp.php?lng=en&amp;Expert=3099</t>
         </is>
       </c>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>Systemic</t>
+        </is>
+      </c>
+      <c r="N182" s="2" t="inlineStr">
+        <is>
+          <t>Antibody</t>
+        </is>
+      </c>
+      <c r="O182" s="2" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="P182" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001183</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001183</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Rheumatoid aortitis</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t>Autoimmune aortitis (isolated, non-vasculitic)</t>
+        </is>
+      </c>
+      <c r="E183" s="4" t="inlineStr"/>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>38877003</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr"/>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>4306357</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr"/>
+      <c r="K183" s="4" t="inlineStr"/>
+      <c r="L183" s="4" t="inlineStr"/>
       <c r="M183" s="2" t="inlineStr">
         <is>
-          <t>Systemic</t>
-        </is>
-      </c>
-      <c r="N183" s="2" t="inlineStr">
-        <is>
-          <t>Antibody</t>
-        </is>
-      </c>
-      <c r="O183" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
+          <t>Vascular system</t>
+        </is>
+      </c>
+      <c r="N183" s="2" t="inlineStr"/>
+      <c r="O183" s="2" t="inlineStr"/>
       <c r="P183" s="2" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001183</t>
+          <t>ARI:0001184</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001183</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001184</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Rheumatoid aortitis</t>
-        </is>
-      </c>
-      <c r="D184" s="4" t="inlineStr">
-        <is>
-          <t>Autoimmune aortitis (isolated, non-vasculitic)</t>
-        </is>
-      </c>
+          <t>Rheumatoid arthritis</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr"/>
       <c r="E184" s="4" t="inlineStr"/>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>38877003</t>
+          <t>69896004</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr"/>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>4306357</t>
-        </is>
-      </c>
-      <c r="I184" s="2" t="inlineStr"/>
+          <t>80809</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>69896004</t>
+        </is>
+      </c>
       <c r="J184" s="2" t="inlineStr"/>
-      <c r="K184" s="4" t="inlineStr"/>
-      <c r="L184" s="4" t="inlineStr"/>
-      <c r="M184" s="2" t="inlineStr">
-        <is>
-          <t>Vascular system</t>
-        </is>
-      </c>
-      <c r="N184" s="2" t="inlineStr"/>
-      <c r="O184" s="2" t="inlineStr"/>
-      <c r="P184" s="2" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001184</t>
-        </is>
-      </c>
-      <c r="B185" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001184</t>
-        </is>
-      </c>
-      <c r="C185" s="2" t="inlineStr">
-        <is>
-          <t>Rheumatoid arthritis</t>
-        </is>
-      </c>
-      <c r="D185" s="4" t="inlineStr"/>
-      <c r="E185" s="4" t="inlineStr"/>
-      <c r="F185" s="3" t="inlineStr">
-        <is>
-          <t>69896004</t>
-        </is>
-      </c>
-      <c r="G185" s="2" t="inlineStr"/>
-      <c r="H185" s="3" t="inlineStr">
-        <is>
-          <t>80809</t>
-        </is>
-      </c>
-      <c r="I185" s="2" t="inlineStr">
-        <is>
-          <t>69896004</t>
-        </is>
-      </c>
-      <c r="J185" s="2" t="inlineStr"/>
-      <c r="K185" s="4" t="inlineStr">
+      <c r="K184" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Rheumatoid arthritis (RA) is an autoimmune disease marked by inflammation and damage to joints, surrounding bone, blood vessels, and connective tissue.   This disorder usually affects both sides of the body (i.e. both ankles or both wrists). It can also damage the lungs, heart, eyes, skin, and various other body systems.    
 Joints affected by RA are often painful, stiff, and swollen, especially in the morning, and symptoms typically appear in flares followed by remission.  Research has not determined the cause of RA but associations have been found with certain genes, infections, and hormonal changes.  Risk also increases with inhalation of hazardous particles in certain occupations and chronic smoking.  
@@ -12243,14 +12191,82 @@
 </t>
         </is>
       </c>
+      <c r="L184" s="4" t="inlineStr">
+        <is>
+          <t>Tuncer 2018; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC6117145/</t>
+        </is>
+      </c>
+      <c r="M184" s="2" t="inlineStr">
+        <is>
+          <t>Musculoskeletal</t>
+        </is>
+      </c>
+      <c r="N184" s="2" t="inlineStr">
+        <is>
+          <t>Antibody</t>
+        </is>
+      </c>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="P184" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001185</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001185</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Rheumatoid vasculitis</t>
+        </is>
+      </c>
+      <c r="D185" s="4" t="inlineStr">
+        <is>
+          <t>RV</t>
+        </is>
+      </c>
+      <c r="E185" s="4" t="inlineStr"/>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>400054000</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr"/>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>4271003</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>400054000</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr"/>
+      <c r="K185" s="4" t="inlineStr">
+        <is>
+          <t>Rheumatoid vasculitis (RV) is a rare autoimmune disorder affecting a small number of patients with rheumatoid arthritis, which causes inflammation and damage to the blood vessels.  Vessels in any part of the body may be affected, though large blood vessels are less likely to be impacted than medium or small blood vessels.  RV most often develops in patients who have suffered from rheumatoid arthritis for 10 to 14 years.  Patients often experience feelings of malaise, sores on the legs, severely decreased blood flow to the fingers and toes, nerve problems, and eye aggravation.  The cause of RV is uncertain, though smoking is believed to significantly increase risk.  Complications involving the organs may be fatal.  Available treatments have mixed success, and prognosis remains poor.</t>
+        </is>
+      </c>
       <c r="L185" s="4" t="inlineStr">
         <is>
-          <t>Tuncer 2018; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC6117145/</t>
+          <t>Bartels 2009; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC2867593/</t>
         </is>
       </c>
       <c r="M185" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal</t>
+          <t>Vascular system</t>
         </is>
       </c>
       <c r="N185" s="2" t="inlineStr">
@@ -12270,115 +12286,47 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001185</t>
+          <t>ARI:0001186</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001185</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001186</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Rheumatoid vasculitis</t>
+          <t>Sarcoidosis</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>RV</t>
-        </is>
-      </c>
-      <c r="E186" s="4" t="inlineStr"/>
+          <t>Besnier-Boeck-Schaumann disease</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t>Lofgrens syndrome; Lupus pernio</t>
+        </is>
+      </c>
       <c r="F186" s="3" t="inlineStr">
         <is>
-          <t>400054000</t>
+          <t>72470008, 238676008, 31541009</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr"/>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>4271003</t>
+          <t>4081069, 4216556, 438688</t>
         </is>
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>400054000</t>
+          <t>72470008, 238676008, 31541009</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr"/>
       <c r="K186" s="4" t="inlineStr">
-        <is>
-          <t>Rheumatoid vasculitis (RV) is a rare autoimmune disorder affecting a small number of patients with rheumatoid arthritis, which causes inflammation and damage to the blood vessels.  Vessels in any part of the body may be affected, though large blood vessels are less likely to be impacted than medium or small blood vessels.  RV most often develops in patients who have suffered from rheumatoid arthritis for 10 to 14 years.  Patients often experience feelings of malaise, sores on the legs, severely decreased blood flow to the fingers and toes, nerve problems, and eye aggravation.  The cause of RV is uncertain, though smoking is believed to significantly increase risk.  Complications involving the organs may be fatal.  Available treatments have mixed success, and prognosis remains poor.</t>
-        </is>
-      </c>
-      <c r="L186" s="4" t="inlineStr">
-        <is>
-          <t>Bartels 2009; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC2867593/</t>
-        </is>
-      </c>
-      <c r="M186" s="2" t="inlineStr">
-        <is>
-          <t>Vascular system</t>
-        </is>
-      </c>
-      <c r="N186" s="2" t="inlineStr">
-        <is>
-          <t>Antibody</t>
-        </is>
-      </c>
-      <c r="O186" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
-      <c r="P186" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001186</t>
-        </is>
-      </c>
-      <c r="B187" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001186</t>
-        </is>
-      </c>
-      <c r="C187" s="2" t="inlineStr">
-        <is>
-          <t>Sarcoidosis</t>
-        </is>
-      </c>
-      <c r="D187" s="4" t="inlineStr">
-        <is>
-          <t>Besnier-Boeck-Schaumann disease</t>
-        </is>
-      </c>
-      <c r="E187" s="4" t="inlineStr">
-        <is>
-          <t>Lofgrens syndrome; Lupus pernio</t>
-        </is>
-      </c>
-      <c r="F187" s="3" t="inlineStr">
-        <is>
-          <t>72470008, 238676008, 31541009</t>
-        </is>
-      </c>
-      <c r="G187" s="2" t="inlineStr"/>
-      <c r="H187" s="3" t="inlineStr">
-        <is>
-          <t>4081069, 4216556, 438688</t>
-        </is>
-      </c>
-      <c r="I187" s="2" t="inlineStr">
-        <is>
-          <t>72470008, 238676008, 31541009</t>
-        </is>
-      </c>
-      <c r="J187" s="2" t="inlineStr"/>
-      <c r="K187" s="4" t="inlineStr">
         <is>
           <t>One way the immune system works is to surround an invader and keep it from harming the body. Those small clumps of immune system cells are called granulomas and they form as part of the body's inflammation response to foreign, potentially harmful, substances. 
 In sarcoidosis the inflammation process gets out of control, and granulomas form even though there is no foreign substance, and the number of granulomas increases. When left untreated, the granulomas harden and produce permanent scars, usually in the lungs but they can occur in other organs and tissues.  
@@ -12386,14 +12334,83 @@
 Sarcoidosis often starts with a set of symptoms collectively referred to as Lofgren's Syndrome (see below).</t>
         </is>
       </c>
+      <c r="L186" s="4" t="inlineStr">
+        <is>
+          <t>Baughman 2016; https://pubmed.ncbi.nlm.nih.gov/27509154/</t>
+        </is>
+      </c>
+      <c r="M186" s="2" t="inlineStr">
+        <is>
+          <t>Systemic</t>
+        </is>
+      </c>
+      <c r="N186" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="P186" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001187</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001187</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Schnitzler syndrome</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t>Chronic urticaria with gammapathy; Chronic urticaria with gammopathy; Chronic urticaria with macroglobulinemia; Schnitzler's syndrome</t>
+        </is>
+      </c>
+      <c r="E187" s="4" t="inlineStr"/>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>402415001</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr"/>
+      <c r="H187" s="3" t="inlineStr">
+        <is>
+          <t>4297647</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>402415001</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr"/>
+      <c r="K187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schnitzler syndrome is a disease in which periodic episodes of inflammation occur. It is considered an autoinflammatory disease, not an autoimmune disease, because the immune system does not mistakenly attack healthy cells. Instead, Schnitzler syndrome is believed to arise from a problem with the immune system itself. It is uncertain what causes Schnitzler syndrome, but it does not appear to be hereditary.
+Patients with Schnitzler syndrome typically experience chronic rash, relapsing fevers, pain and inflammation in the joints, enlarged lymph nodes, and an excess of certain proteins in the blood.  The condition is chronic, generally without worsening, though 10-15% of people with Schnitzler syndrome experience cancerous or non-cancerous overproduction of certain types of white blood cells. There is no cure, but treatments may relieve symptoms in some individuals.   </t>
+        </is>
+      </c>
       <c r="L187" s="4" t="inlineStr">
         <is>
-          <t>Baughman 2016; https://pubmed.ncbi.nlm.nih.gov/27509154/</t>
+          <t>de Koning 2014; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4405827/</t>
         </is>
       </c>
       <c r="M187" s="2" t="inlineStr">
         <is>
-          <t>Systemic</t>
+          <t>Musculoskeletal</t>
         </is>
       </c>
       <c r="N187" s="2" t="inlineStr">
@@ -12413,56 +12430,51 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001187</t>
+          <t>ARI:0001188</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001187</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001188</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Schnitzler syndrome</t>
-        </is>
-      </c>
-      <c r="D188" s="4" t="inlineStr">
-        <is>
-          <t>Chronic urticaria with gammapathy; Chronic urticaria with gammopathy; Chronic urticaria with macroglobulinemia; Schnitzler's syndrome</t>
-        </is>
-      </c>
+          <t>Scleritis</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr"/>
       <c r="E188" s="4" t="inlineStr"/>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>402415001</t>
+          <t>78370002</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr"/>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>4297647</t>
+          <t>434944</t>
         </is>
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>402415001</t>
+          <t>78370002</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr"/>
       <c r="K188" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Schnitzler syndrome is a disease in which periodic episodes of inflammation occur. It is considered an autoinflammatory disease, not an autoimmune disease, because the immune system does not mistakenly attack healthy cells. Instead, Schnitzler syndrome is believed to arise from a problem with the immune system itself. It is uncertain what causes Schnitzler syndrome, but it does not appear to be hereditary.
-Patients with Schnitzler syndrome typically experience chronic rash, relapsing fevers, pain and inflammation in the joints, enlarged lymph nodes, and an excess of certain proteins in the blood.  The condition is chronic, generally without worsening, though 10-15% of people with Schnitzler syndrome experience cancerous or non-cancerous overproduction of certain types of white blood cells. There is no cure, but treatments may relieve symptoms in some individuals.   </t>
+          <t xml:space="preserve">Scleritis is an inflammation of the white tissue, the sclera, that surrounds most of the eye. Though scleritis is a symptom of a number of autoimmune diseases, it is suspected of being an autoimmune disease itself.  </t>
         </is>
       </c>
       <c r="L188" s="4" t="inlineStr">
         <is>
-          <t>de Koning 2014; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC4405827/</t>
+          <t>Honik 2013; https://pubmed.ncbi.nlm.nih.gov/24145628/</t>
         </is>
       </c>
       <c r="M188" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal</t>
+          <t>Eye</t>
         </is>
       </c>
       <c r="N188" s="2" t="inlineStr">
@@ -12482,61 +12494,65 @@
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001188</t>
+          <t>ARI:0001189</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001188</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001189</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Scleritis</t>
-        </is>
-      </c>
-      <c r="D189" s="4" t="inlineStr"/>
+          <t>Sjögren's disease</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>Keratoconjunctivitis sicca; Sicca syndrome; Sjogren's disease; Sjögrens disease; Sjögren's syndrome; SJS</t>
+        </is>
+      </c>
       <c r="E189" s="4" t="inlineStr"/>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>78370002</t>
+          <t>83901003</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr"/>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>434944</t>
+          <t>254443</t>
         </is>
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>78370002</t>
+          <t>83901003</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr"/>
       <c r="K189" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scleritis is an inflammation of the white tissue, the sclera, that surrounds most of the eye. Though scleritis is a symptom of a number of autoimmune diseases, it is suspected of being an autoimmune disease itself.  </t>
+          <t xml:space="preserve">Sicca syndrome is marked by dry mouth and dry eyes. If these symptoms are caused by an autoimmune process, it is called Sjogren's disease. See &lt;a href="/Disease_Profile/Sj%C3%B6grens-disease.aspx"&gt;Sjögrens disease for more information. </t>
         </is>
       </c>
       <c r="L189" s="4" t="inlineStr">
         <is>
-          <t>Honik 2013; https://pubmed.ncbi.nlm.nih.gov/24145628/</t>
+          <t>Narváez 2020; https://pubmed.ncbi.nlm.nih.gov/32606345/</t>
         </is>
       </c>
       <c r="M189" s="2" t="inlineStr">
         <is>
-          <t>Eye</t>
+          <t>Glands</t>
         </is>
       </c>
       <c r="N189" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Antibody</t>
         </is>
       </c>
       <c r="O189" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P189" s="2" t="n">
@@ -12546,55 +12562,55 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001189</t>
+          <t>ARI:0001190</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001189</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001190</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Sjögren's disease</t>
+          <t>SLE glomerulonephritis syndrome</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
         <is>
-          <t>Keratoconjunctivitis sicca; Sicca syndrome; Sjogren's disease; Sjögrens disease; Sjögren's syndrome; SJS</t>
+          <t>Lupus nephritis</t>
         </is>
       </c>
       <c r="E190" s="4" t="inlineStr"/>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>83901003</t>
+          <t>68815009</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr"/>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>254443</t>
+          <t>4285717</t>
         </is>
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>83901003</t>
+          <t>68815009</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr"/>
       <c r="K190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sicca syndrome is marked by dry mouth and dry eyes. If these symptoms are caused by an autoimmune process, it is called Sjogren's disease. See &lt;a href="/Disease_Profile/Sj%C3%B6grens-disease.aspx"&gt;Sjögrens disease for more information. </t>
+          <t>Lupus nephritis is a complication in patients with systemic lupus erythematosus (SLE), an autoimmune condition causing inflammation of the body's tissues.  Lupus nephritis targets the kidneys, causing damage and inflammation, which prevents normal function and may lead to kidney failure.  Significant delay or lack of treatment can be fatal, but early medical care can manage symptoms and result in a good prognosis.</t>
         </is>
       </c>
       <c r="L190" s="4" t="inlineStr">
         <is>
-          <t>Narváez 2020; https://pubmed.ncbi.nlm.nih.gov/32606345/</t>
+          <t>Wang 2017; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC5864167/</t>
         </is>
       </c>
       <c r="M190" s="2" t="inlineStr">
         <is>
-          <t>Glands</t>
+          <t>Kidney</t>
         </is>
       </c>
       <c r="N190" s="2" t="inlineStr">
@@ -12614,112 +12630,104 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001190</t>
+          <t>ARI:0001191</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001190</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001191</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>SLE glomerulonephritis syndrome</t>
-        </is>
-      </c>
-      <c r="D191" s="4" t="inlineStr">
-        <is>
-          <t>Lupus nephritis</t>
-        </is>
-      </c>
-      <c r="E191" s="4" t="inlineStr"/>
+          <t>Small fiber neuropathy</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr"/>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>Autoimmune small fiber neuropathy</t>
+        </is>
+      </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>68815009</t>
+          <t>709489006</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr"/>
       <c r="H191" s="3" t="inlineStr">
         <is>
-          <t>4285717</t>
-        </is>
-      </c>
-      <c r="I191" s="2" t="inlineStr">
-        <is>
-          <t>68815009</t>
-        </is>
-      </c>
+          <t>46271378</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr"/>
       <c r="J191" s="2" t="inlineStr"/>
-      <c r="K191" s="4" t="inlineStr">
-        <is>
-          <t>Lupus nephritis is a complication in patients with systemic lupus erythematosus (SLE), an autoimmune condition causing inflammation of the body's tissues.  Lupus nephritis targets the kidneys, causing damage and inflammation, which prevents normal function and may lead to kidney failure.  Significant delay or lack of treatment can be fatal, but early medical care can manage symptoms and result in a good prognosis.</t>
-        </is>
+      <c r="K191" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="L191" s="4" t="inlineStr">
         <is>
-          <t>Wang 2017; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC5864167/</t>
+          <t>1 million</t>
         </is>
       </c>
       <c r="M191" s="2" t="inlineStr">
         <is>
-          <t>Kidney</t>
-        </is>
-      </c>
-      <c r="N191" s="2" t="inlineStr">
-        <is>
-          <t>Antibody</t>
-        </is>
-      </c>
-      <c r="O191" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
+          <t>Nervous System</t>
+        </is>
+      </c>
+      <c r="N191" s="2" t="inlineStr"/>
+      <c r="O191" s="2" t="inlineStr"/>
       <c r="P191" s="2" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001191</t>
+          <t>ARI:0001192</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001191</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001192</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Small fiber neuropathy</t>
-        </is>
-      </c>
-      <c r="D192" s="4" t="inlineStr"/>
-      <c r="E192" s="4" t="inlineStr">
-        <is>
-          <t>Autoimmune small fiber neuropathy</t>
-        </is>
-      </c>
+          <t>Steroid-responsive encephalopathy associated with autoimmune thyroiditis</t>
+        </is>
+      </c>
+      <c r="D192" s="4" t="inlineStr">
+        <is>
+          <t>Encephalopathy associated with autoimmune thyroid disease; Hashimoto's encephalitis; Hashimoto's encephalopathy; Nonvasculitic autoimmune meningoecephalitis</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr"/>
       <c r="F192" s="3" t="inlineStr">
         <is>
-          <t>709489006</t>
+          <t>771271000</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr"/>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>46271378</t>
-        </is>
-      </c>
-      <c r="I192" s="2" t="inlineStr"/>
+          <t>36674282</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>771271000</t>
+        </is>
+      </c>
       <c r="J192" s="2" t="inlineStr"/>
-      <c r="K192" s="4" t="n">
-        <v>1</v>
+      <c r="K192" s="4" t="inlineStr">
+        <is>
+          <t>Steroid-responsive encephalopathy associated with autoimmune thyroiditis (SREAT), often called Hashimoto’s encephalopathy, is a rare autoimmune disease that affects both the nervous system and endocrine system. Encephalopathy, or brain dysfunction, resulting from thyroid disease can lead to muscle twitches, seizures, confusion, and even paranoia. The three forms of SREAT are acute, subacute, and chronic. SREAT also ranges in severity, from mild cognitive impairment to life-threatening seizures.</t>
+        </is>
       </c>
       <c r="L192" s="4" t="inlineStr">
         <is>
-          <t>1 million</t>
+          <t>Mocellin 2007; https://pubmed.ncbi.nlm.nih.gov/17850170/</t>
         </is>
       </c>
       <c r="M192" s="2" t="inlineStr">
@@ -12727,64 +12735,72 @@
           <t>Nervous System</t>
         </is>
       </c>
-      <c r="N192" s="2" t="inlineStr"/>
-      <c r="O192" s="2" t="inlineStr"/>
+      <c r="N192" s="2" t="inlineStr">
+        <is>
+          <t>Antibody</t>
+        </is>
+      </c>
+      <c r="O192" s="2" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
       <c r="P192" s="2" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001192</t>
+          <t>ARI:0001193</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001192</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001193</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Steroid-responsive encephalopathy associated with autoimmune thyroiditis</t>
+          <t>Stiff-person syndrome</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
         <is>
-          <t>Encephalopathy associated with autoimmune thyroid disease; Hashimoto's encephalitis; Hashimoto's encephalopathy; Nonvasculitic autoimmune meningoecephalitis</t>
+          <t>Moersch-Woltman syndrome; Stiff man syndrome; Stiff person syndrome</t>
         </is>
       </c>
       <c r="E193" s="4" t="inlineStr"/>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>771271000</t>
+          <t>5217008</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr"/>
       <c r="H193" s="3" t="inlineStr">
         <is>
-          <t>36674282</t>
+          <t>379008</t>
         </is>
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>771271000</t>
+          <t>5217008</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr"/>
       <c r="K193" s="4" t="inlineStr">
         <is>
-          <t>Steroid-responsive encephalopathy associated with autoimmune thyroiditis (SREAT), often called Hashimoto’s encephalopathy, is a rare autoimmune disease that affects both the nervous system and endocrine system. Encephalopathy, or brain dysfunction, resulting from thyroid disease can lead to muscle twitches, seizures, confusion, and even paranoia. The three forms of SREAT are acute, subacute, and chronic. SREAT also ranges in severity, from mild cognitive impairment to life-threatening seizures.</t>
+          <t>Stiff person syndrome (SPS) is a rare, progressive syndrome believed to be autoimmune in nature, though the cause is currently unknown.  SPS is characterized by decreased inhibition of the central nervous system, which leads to greater muscle activity causing flares of severe stiffness and spasms, usually in the muscles of the trunk and limbs.  Triggers include noise, touch, and emotional distress.  SPS may result in disability, fractures due to severe muscle contractions, and abnormal posture.  Comorbidities may include diabetes, thyroiditis, vitiligo, and pernicious anemia.  There is no cure, but symptoms can be managed through treatment.</t>
         </is>
       </c>
       <c r="L193" s="4" t="inlineStr">
         <is>
-          <t>Mocellin 2007; https://pubmed.ncbi.nlm.nih.gov/17850170/</t>
+          <t>Nguyen 2019; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC6944797/</t>
         </is>
       </c>
       <c r="M193" s="2" t="inlineStr">
         <is>
-          <t>Nervous System</t>
+          <t>Musculoskeletal</t>
         </is>
       </c>
       <c r="N193" s="2" t="inlineStr">
@@ -12804,135 +12820,136 @@
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001193</t>
+          <t>ARI:0001194</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001193</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001194</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Stiff-person syndrome</t>
+          <t>Subacute bacterial endocarditis</t>
         </is>
       </c>
       <c r="D194" s="4" t="inlineStr">
         <is>
-          <t>Moersch-Woltman syndrome; Stiff man syndrome; Stiff person syndrome</t>
+          <t>Subacute infective endocarditis; Subacute native valve endocarditis</t>
         </is>
       </c>
       <c r="E194" s="4" t="inlineStr"/>
       <c r="F194" s="3" t="inlineStr">
         <is>
-          <t>5217008</t>
+          <t>73774007</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr"/>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>379008</t>
+          <t>4249899</t>
         </is>
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>5217008</t>
+          <t>73774007</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr"/>
       <c r="K194" s="4" t="inlineStr">
-        <is>
-          <t>Stiff person syndrome (SPS) is a rare, progressive syndrome believed to be autoimmune in nature, though the cause is currently unknown.  SPS is characterized by decreased inhibition of the central nervous system, which leads to greater muscle activity causing flares of severe stiffness and spasms, usually in the muscles of the trunk and limbs.  Triggers include noise, touch, and emotional distress.  SPS may result in disability, fractures due to severe muscle contractions, and abnormal posture.  Comorbidities may include diabetes, thyroiditis, vitiligo, and pernicious anemia.  There is no cure, but symptoms can be managed through treatment.</t>
-        </is>
-      </c>
-      <c r="L194" s="4" t="inlineStr">
-        <is>
-          <t>Nguyen 2019; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC6944797/</t>
-        </is>
-      </c>
-      <c r="M194" s="2" t="inlineStr">
-        <is>
-          <t>Musculoskeletal</t>
-        </is>
-      </c>
-      <c r="N194" s="2" t="inlineStr">
-        <is>
-          <t>Antibody</t>
-        </is>
-      </c>
-      <c r="O194" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
-      <c r="P194" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001194</t>
-        </is>
-      </c>
-      <c r="B195" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001194</t>
-        </is>
-      </c>
-      <c r="C195" s="2" t="inlineStr">
-        <is>
-          <t>Subacute bacterial endocarditis</t>
-        </is>
-      </c>
-      <c r="D195" s="4" t="inlineStr">
-        <is>
-          <t>Subacute infective endocarditis; Subacute native valve endocarditis</t>
-        </is>
-      </c>
-      <c r="E195" s="4" t="inlineStr"/>
-      <c r="F195" s="3" t="inlineStr">
-        <is>
-          <t>73774007</t>
-        </is>
-      </c>
-      <c r="G195" s="2" t="inlineStr"/>
-      <c r="H195" s="3" t="inlineStr">
-        <is>
-          <t>4249899</t>
-        </is>
-      </c>
-      <c r="I195" s="2" t="inlineStr">
-        <is>
-          <t>73774007</t>
-        </is>
-      </c>
-      <c r="J195" s="2" t="inlineStr"/>
-      <c r="K195" s="4" t="inlineStr">
         <is>
           <t>Subacute bacterial endocarditis (SBE) is a type of bacterial endocarditis. Endocarditis is an infection of the inner lining of your heart chambers and heart valves (the endocardium).  In SBE, the lining inside the heart valves become infected. 
 SBE is not an autoimmune disease, but patients are at increased risk of developing autoimmune disease following SBE. 
 This condition most frequently occurs following surgery to a region of the body infected with streptococcal bacteria.  Invasive surgery in the infected tissue facilitates the spread of the bacteria to the heart valves by way of the blood.  The infection normally develops slowly during the two weeks after surgery and may persist for months.  SBE typically only occurs in patients who already have damage to their heart valves from other health conditions.  SBE is difficult to diagnosis because initial symptoms consist almost exclusively of feelings of malaise, which are also common in many other disorders.  SBE may trigger the onset of autoimmune conditions, such as vasculitis. If left untreated, complications can be fatal; however, positive outcomes are expected with early medical care.</t>
         </is>
       </c>
+      <c r="L194" s="4" t="inlineStr">
+        <is>
+          <t>Cahill 2017; https://pubmed.ncbi.nlm.nih.gov/28104075/</t>
+        </is>
+      </c>
+      <c r="M194" s="2" t="inlineStr">
+        <is>
+          <t>Heart</t>
+        </is>
+      </c>
+      <c r="N194" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="O194" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="P194" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001195</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001195</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>Sympathetic uveitis</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>Exciting Eye; Spared Eye Injury; Sympathetic ophthalmia; Sympathizing Eye</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="inlineStr"/>
+      <c r="F195" s="3" t="inlineStr">
+        <is>
+          <t>75315001</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr"/>
+      <c r="H195" s="3" t="inlineStr">
+        <is>
+          <t>438739</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>75315001</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr"/>
+      <c r="K195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sympathetic Ophthalmia (SO) is a rare inflammatory condition that affects both eyes following trauma or surgery to one of the eyes. The immune system is sensitized to proteins from the damaged eye and then attacks those same proteins in the uninjured (or “spared” eye), leading to inflammation of the uninjured eye. Sympathetic ophthalmia is a form of uveitis. The disease can lead to blindness. 
+</t>
+        </is>
+      </c>
       <c r="L195" s="4" t="inlineStr">
         <is>
-          <t>Cahill 2017; https://pubmed.ncbi.nlm.nih.gov/28104075/</t>
+          <t>Arevalo 2012; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC3277011/</t>
         </is>
       </c>
       <c r="M195" s="2" t="inlineStr">
         <is>
-          <t>Heart</t>
+          <t>Eye</t>
         </is>
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Antibody</t>
         </is>
       </c>
       <c r="O195" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P195" s="2" t="n">
@@ -12942,56 +12959,55 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001195</t>
+          <t>ARI:0001196</t>
         </is>
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001195</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001196</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Sympathetic uveitis</t>
+          <t>Systemic lupus erythematosus</t>
         </is>
       </c>
       <c r="D196" s="4" t="inlineStr">
         <is>
-          <t>Exciting Eye; Spared Eye Injury; Sympathetic ophthalmia; Sympathizing Eye</t>
+          <t>Lupus; SLE</t>
         </is>
       </c>
       <c r="E196" s="4" t="inlineStr"/>
       <c r="F196" s="3" t="inlineStr">
         <is>
-          <t>75315001</t>
+          <t>55464009</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr"/>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>438739</t>
+          <t>257628, 255891</t>
         </is>
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>75315001</t>
+          <t>55464009</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr"/>
       <c r="K196" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sympathetic Ophthalmia (SO) is a rare inflammatory condition that affects both eyes following trauma or surgery to one of the eyes. The immune system is sensitized to proteins from the damaged eye and then attacks those same proteins in the uninjured (or “spared” eye), leading to inflammation of the uninjured eye. Sympathetic ophthalmia is a form of uveitis. The disease can lead to blindness. 
-</t>
+          <t>SLE, the most common type of lupus, is a chronic inflammatory disease that occurs when the body's immune system attacks its own tissues and organs. Inflammation caused by lupus can affect many different body systems — including joints, skin, kidneys, blood cells, brain, heart and lungs.</t>
         </is>
       </c>
       <c r="L196" s="4" t="inlineStr">
         <is>
-          <t>Arevalo 2012; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC3277011/</t>
+          <t>Izmirly 2021; https://pubmed.ncbi.nlm.nih.gov/33474834/</t>
         </is>
       </c>
       <c r="M196" s="2" t="inlineStr">
         <is>
-          <t>Eye</t>
+          <t>Systemic</t>
         </is>
       </c>
       <c r="N196" s="2" t="inlineStr">
@@ -13011,50 +13027,47 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001196</t>
+          <t>ARI:0001197</t>
         </is>
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001196</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001197</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Systemic lupus erythematosus</t>
-        </is>
-      </c>
-      <c r="D197" s="4" t="inlineStr">
-        <is>
-          <t>Lupus; SLE</t>
-        </is>
-      </c>
+          <t>Systemic mast cell disease</t>
+        </is>
+      </c>
+      <c r="D197" s="4" t="inlineStr"/>
       <c r="E197" s="4" t="inlineStr"/>
       <c r="F197" s="3" t="inlineStr">
         <is>
-          <t>55464009</t>
+          <t>397016004</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr"/>
       <c r="H197" s="3" t="inlineStr">
         <is>
-          <t>257628, 255891</t>
+          <t>4246284</t>
         </is>
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>55464009</t>
+          <t>397016004</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr"/>
       <c r="K197" s="4" t="inlineStr">
         <is>
-          <t>SLE, the most common type of lupus, is a chronic inflammatory disease that occurs when the body's immune system attacks its own tissues and organs. Inflammation caused by lupus can affect many different body systems — including joints, skin, kidneys, blood cells, brain, heart and lungs.</t>
+          <t>Systemic mastocytosis is caused when too many mast cells accumulate in the body. It is not an autoimmune disease, but a disease of the immune system, specifically mast cells. Mast cells transport histamine, which is involved in allergic responses.  
+When mastocytosis is limited to the skin, it is called cutaneous mastocytosis, and is a less severe form of the disease.</t>
         </is>
       </c>
       <c r="L197" s="4" t="inlineStr">
         <is>
-          <t>Izmirly 2021; https://pubmed.ncbi.nlm.nih.gov/33474834/</t>
+          <t>Jørgensen 2025; https://pmc.ncbi.nlm.nih.gov/articles/PMC11799073/</t>
         </is>
       </c>
       <c r="M197" s="2" t="inlineStr">
@@ -13064,12 +13077,12 @@
       </c>
       <c r="N197" s="2" t="inlineStr">
         <is>
-          <t>Antibody</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="O197" s="2" t="inlineStr">
         <is>
-          <t>Autoimmune</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="P197" s="2" t="n">
@@ -13079,47 +13092,50 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001197</t>
+          <t>ARI:0001198</t>
         </is>
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001197</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001198</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Systemic mast cell disease</t>
-        </is>
-      </c>
-      <c r="D198" s="4" t="inlineStr"/>
+          <t>Systemic sclerosis</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>Diffuse Systemic sclerosis; Scleroderma; Systemic scleroderma</t>
+        </is>
+      </c>
       <c r="E198" s="4" t="inlineStr"/>
       <c r="F198" s="3" t="inlineStr">
         <is>
-          <t>397016004</t>
+          <t>89155008</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr"/>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>4246284</t>
+          <t>134442</t>
         </is>
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>397016004</t>
+          <t>89155008</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr"/>
       <c r="K198" s="4" t="inlineStr">
         <is>
-          <t>Systemic mastocytosis is caused when too many mast cells accumulate in the body. It is not an autoimmune disease, but a disease of the immune system, specifically mast cells. Mast cells transport histamine, which is involved in allergic responses.  
-When mastocytosis is limited to the skin, it is called cutaneous mastocytosis, and is a less severe form of the disease.</t>
+          <t>Scleroderma is an autoimmune, rheumatic, and chronic disease that affects the body by hardening connective tissue. This disease may also cause issues in the blood vessels, organs, and digestive tract. Scleroderma is characterized as limited or diffuse, referring to the degree of skin involvement, but can both involve any vascular or organ symptoms. These symptoms occur when the body produces too much collagen, which builds up the body’s connective tissues. People who usually get scleroderma are those between the ages of 30 and 50 and tend to be female at birth.</t>
         </is>
       </c>
       <c r="L198" s="4" t="inlineStr">
         <is>
-          <t>Jørgensen 2025; https://pmc.ncbi.nlm.nih.gov/articles/PMC11799073/</t>
+          <t>Barnes 2012; https://pubmed.ncbi.nlm.nih.gov/22269658/</t>
         </is>
       </c>
       <c r="M198" s="2" t="inlineStr">
@@ -13129,12 +13145,12 @@
       </c>
       <c r="N198" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Antibody</t>
         </is>
       </c>
       <c r="O198" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P198" s="2" t="n">
@@ -13144,115 +13160,47 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001198</t>
+          <t>ARI:0001199</t>
         </is>
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001198</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001199</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Systemic sclerosis</t>
+          <t>Systemic sclerosis with limited cutaneous involvement</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
         <is>
-          <t>Diffuse Systemic sclerosis; Scleroderma; Systemic scleroderma</t>
-        </is>
-      </c>
-      <c r="E199" s="4" t="inlineStr"/>
+          <t>CREST syndrome; dcSSc; lcSSc</t>
+        </is>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>Diffuse cutaneous systemic sclerosis; Limited cutaneous systemic sclerosis; Systemic sclerosis sine scleroderma</t>
+        </is>
+      </c>
       <c r="F199" s="3" t="inlineStr">
         <is>
-          <t>89155008</t>
+          <t>298285004, 31848007, 128461001</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr"/>
       <c r="H199" s="3" t="inlineStr">
         <is>
-          <t>134442</t>
+          <t>4185187, 4135937, 4027230</t>
         </is>
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>89155008</t>
+          <t>298285004, 31848007, 128461001</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr"/>
       <c r="K199" s="4" t="inlineStr">
-        <is>
-          <t>Scleroderma is an autoimmune, rheumatic, and chronic disease that affects the body by hardening connective tissue. This disease may also cause issues in the blood vessels, organs, and digestive tract. Scleroderma is characterized as limited or diffuse, referring to the degree of skin involvement, but can both involve any vascular or organ symptoms. These symptoms occur when the body produces too much collagen, which builds up the body’s connective tissues. People who usually get scleroderma are those between the ages of 30 and 50 and tend to be female at birth.</t>
-        </is>
-      </c>
-      <c r="L199" s="4" t="inlineStr">
-        <is>
-          <t>Barnes 2012; https://pubmed.ncbi.nlm.nih.gov/22269658/</t>
-        </is>
-      </c>
-      <c r="M199" s="2" t="inlineStr">
-        <is>
-          <t>Systemic</t>
-        </is>
-      </c>
-      <c r="N199" s="2" t="inlineStr">
-        <is>
-          <t>Antibody</t>
-        </is>
-      </c>
-      <c r="O199" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
-      <c r="P199" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001199</t>
-        </is>
-      </c>
-      <c r="B200" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001199</t>
-        </is>
-      </c>
-      <c r="C200" s="2" t="inlineStr">
-        <is>
-          <t>Systemic sclerosis with limited cutaneous involvement</t>
-        </is>
-      </c>
-      <c r="D200" s="4" t="inlineStr">
-        <is>
-          <t>CREST syndrome; dcSSc; lcSSc</t>
-        </is>
-      </c>
-      <c r="E200" s="4" t="inlineStr">
-        <is>
-          <t>Diffuse cutaneous systemic sclerosis; Limited cutaneous systemic sclerosis; Systemic sclerosis sine scleroderma</t>
-        </is>
-      </c>
-      <c r="F200" s="3" t="inlineStr">
-        <is>
-          <t>298285004, 31848007, 128461001</t>
-        </is>
-      </c>
-      <c r="G200" s="2" t="inlineStr"/>
-      <c r="H200" s="3" t="inlineStr">
-        <is>
-          <t>4185187, 4135937, 4027230</t>
-        </is>
-      </c>
-      <c r="I200" s="2" t="inlineStr">
-        <is>
-          <t>298285004, 31848007, 128461001</t>
-        </is>
-      </c>
-      <c r="J200" s="2" t="inlineStr"/>
-      <c r="K200" s="4" t="inlineStr">
         <is>
           <t>CREST is a subtype of scleroderma, a connective tissue disease characterized by changes in the skin, blood vessels, skeletal muscles, and internal organs. CREST is the acronym for the clinical features seen in individuals with the disease :                        
 C - Calcinosis: calcium deposits in the connective tissues
@@ -13263,79 +13211,147 @@
 To be diagnosed with CREST, you must have 3 out of the 5 symptoms.</t>
         </is>
       </c>
-      <c r="L200" s="4" t="inlineStr">
+      <c r="L199" s="4" t="inlineStr">
         <is>
           <t>Efrimescu 2023; https://pubmed.ncbi.nlm.nih.gov/36686888/</t>
         </is>
       </c>
-      <c r="M200" s="2" t="inlineStr">
+      <c r="M199" s="2" t="inlineStr">
         <is>
           <t>Systemic</t>
         </is>
       </c>
-      <c r="N200" s="2" t="inlineStr">
+      <c r="N199" s="2" t="inlineStr">
         <is>
           <t>Antibody Suspected</t>
         </is>
       </c>
-      <c r="O200" s="2" t="inlineStr">
+      <c r="O199" s="2" t="inlineStr">
         <is>
           <t>Autoimmune</t>
         </is>
       </c>
-      <c r="P200" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="2" t="inlineStr">
+      <c r="P199" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
         <is>
           <t>ARI:0001200</t>
         </is>
       </c>
-      <c r="B201" s="3" t="inlineStr">
+      <c r="B200" s="3" t="inlineStr">
         <is>
           <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001200</t>
         </is>
       </c>
-      <c r="C201" s="2" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr">
         <is>
           <t>Takayasu's arteritis</t>
         </is>
       </c>
-      <c r="D201" s="4" t="inlineStr">
+      <c r="D200" s="4" t="inlineStr">
         <is>
           <t>Takayasu's disease</t>
         </is>
       </c>
-      <c r="E201" s="4" t="inlineStr"/>
-      <c r="F201" s="3" t="inlineStr">
+      <c r="E200" s="4" t="inlineStr"/>
+      <c r="F200" s="3" t="inlineStr">
         <is>
           <t>359789008</t>
         </is>
       </c>
-      <c r="G201" s="2" t="inlineStr"/>
-      <c r="H201" s="3" t="inlineStr">
+      <c r="G200" s="2" t="inlineStr"/>
+      <c r="H200" s="3" t="inlineStr">
         <is>
           <t>440740</t>
         </is>
       </c>
-      <c r="I201" s="2" t="inlineStr">
+      <c r="I200" s="2" t="inlineStr">
         <is>
           <t>359789008</t>
         </is>
       </c>
-      <c r="J201" s="2" t="inlineStr"/>
-      <c r="K201" s="4" t="inlineStr">
+      <c r="J200" s="2" t="inlineStr"/>
+      <c r="K200" s="4" t="inlineStr">
         <is>
           <t>Takayasu’s arteritis (TA) is a rare disease that affects large blood vessels, especially the aorta and its major branches. It is sometimes called "pulseless disease" because it can weaken or block pulses in the arms and legs. The condition mainly affects young women, particularly those from Asian and South American countries. Although it is most common in women under 40, TA can also occur in men and older individuals. 
 In Takayasu’s arteritis, inflammation causes the walls of affected arteries to become thickened and scarred, which can reduce blood flow to important organs and limbs. The disease is marked by patches of severe inflammation in the artery walls, often alternating with areas of normal tissue. Over time, the arteries can become narrowed (stenosis) or, in some cases, develop bulges (aneurysms). The aortic wall is often involved, with inflammatory cells such as lymphocytes and plasma cells attacking the outermost layers of the artery and sometimes extending into the surrounding tissues. 
 Early symptoms may include fever, night sweats, fatigue, joint pain, and chest discomfort. As the disease progresses, inflammation and damage to major arteries can lead to headaches, dizziness, vision problems, and even fainting due to reduced blood flow to the brain. Narrowing of the arteries supplying the arms and upper body can cause pain and weakness, while involvement of the coronary arteries can result in chest pain and an increased risk of heart disease, including aortic regurgitation, a serious condition that allows blood to flow backward into the heart and can lead to heart failure.</t>
         </is>
       </c>
+      <c r="L200" s="4" t="inlineStr">
+        <is>
+          <t>Watts 2009; https://pubmed.ncbi.nlm.nih.gov/19542212/</t>
+        </is>
+      </c>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>Vascular system</t>
+        </is>
+      </c>
+      <c r="N200" s="2" t="inlineStr">
+        <is>
+          <t>TCELL</t>
+        </is>
+      </c>
+      <c r="O200" s="2" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="P200" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001201</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001201</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>Temporal arteritis</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>Cranial arteritis; GCA; Giant cell arteritis; Granulomatous arteritis; Horton's disease</t>
+        </is>
+      </c>
+      <c r="E201" s="4" t="inlineStr"/>
+      <c r="F201" s="3" t="inlineStr">
+        <is>
+          <t>400130008</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr"/>
+      <c r="H201" s="3" t="inlineStr">
+        <is>
+          <t>4290976</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>400130008</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr"/>
+      <c r="K201" s="4" t="inlineStr">
+        <is>
+          <t>Temporal arteritis, also known as giant cell arteritis, is an inflammation of the lining of the arteries that typically affects the arteries in the head. Temporal arteritis can frequently cause headaches, scalp tenderness, jaw pain and vision problems.</t>
+        </is>
+      </c>
       <c r="L201" s="4" t="inlineStr">
         <is>
-          <t>Watts 2009; https://pubmed.ncbi.nlm.nih.gov/19542212/</t>
+          <t>Crowson 2017; https://pubmed.ncbi.nlm.nih.gov/28551169/</t>
         </is>
       </c>
       <c r="M201" s="2" t="inlineStr">
@@ -13360,177 +13376,177 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001201</t>
+          <t>ARI:0001202</t>
         </is>
       </c>
       <c r="B202" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001201</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001202</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Temporal arteritis</t>
+          <t>TIF1-gamma positive dermatomyositis</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
         <is>
-          <t>Cranial arteritis; GCA; Giant cell arteritis; Granulomatous arteritis; Horton's disease</t>
+          <t>Cancer-associated myositis</t>
         </is>
       </c>
       <c r="E202" s="4" t="inlineStr"/>
-      <c r="F202" s="3" t="inlineStr">
-        <is>
-          <t>400130008</t>
-        </is>
-      </c>
+      <c r="F202" s="2" t="inlineStr"/>
       <c r="G202" s="2" t="inlineStr"/>
-      <c r="H202" s="3" t="inlineStr">
-        <is>
-          <t>4290976</t>
-        </is>
-      </c>
-      <c r="I202" s="2" t="inlineStr">
-        <is>
-          <t>400130008</t>
-        </is>
-      </c>
-      <c r="J202" s="2" t="inlineStr"/>
-      <c r="K202" s="4" t="inlineStr">
-        <is>
-          <t>Temporal arteritis, also known as giant cell arteritis, is an inflammation of the lining of the arteries that typically affects the arteries in the head. Temporal arteritis can frequently cause headaches, scalp tenderness, jaw pain and vision problems.</t>
-        </is>
-      </c>
-      <c r="L202" s="4" t="inlineStr">
-        <is>
-          <t>Crowson 2017; https://pubmed.ncbi.nlm.nih.gov/28551169/</t>
-        </is>
-      </c>
+      <c r="H202" s="2" t="inlineStr"/>
+      <c r="I202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed No Code</t>
+        </is>
+      </c>
+      <c r="K202" s="4" t="inlineStr"/>
+      <c r="L202" s="4" t="inlineStr"/>
       <c r="M202" s="2" t="inlineStr">
         <is>
-          <t>Vascular system</t>
-        </is>
-      </c>
-      <c r="N202" s="2" t="inlineStr">
-        <is>
-          <t>TCELL</t>
-        </is>
-      </c>
-      <c r="O202" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
+          <t>Systemic</t>
+        </is>
+      </c>
+      <c r="N202" s="2" t="inlineStr"/>
+      <c r="O202" s="2" t="inlineStr"/>
       <c r="P202" s="2" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001202</t>
+          <t>ARI:0001203</t>
         </is>
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001202</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001203</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>TIF1-gamma positive dermatomyositis</t>
+          <t>Tolosa-Hunt syndrome</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
         <is>
-          <t>Cancer-associated myositis</t>
+          <t>Non-specific inflammation of the cavernous sinus; Non-specific inflammation of the superior orbital fissure; Painful Ophthalmoplegia; THS</t>
         </is>
       </c>
       <c r="E203" s="4" t="inlineStr"/>
-      <c r="F203" s="2" t="inlineStr"/>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>95794005</t>
+        </is>
+      </c>
       <c r="G203" s="2" t="inlineStr"/>
-      <c r="H203" s="2" t="inlineStr"/>
-      <c r="I203" s="2" t="inlineStr"/>
-      <c r="J203" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed No Code</t>
-        </is>
-      </c>
-      <c r="K203" s="4" t="inlineStr"/>
-      <c r="L203" s="4" t="inlineStr"/>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>4317989</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>95794005</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr"/>
+      <c r="K203" s="4" t="inlineStr">
+        <is>
+          <t>Patients with Tolosa-Hunt syndrome experience episodes of severe headaches surrounding the eyes, along with restricted eye movement that is painful (ophthalmoplegia). Normally, only one eye is affected and will frequently appear protruded. Symptoms may also include nerve abnormalities, such as eyelid drooping, double vision, large pupil, and numbness of the face. This disorder typically occurs in relapsing flares. The cause of Tolosa-Hunt syndrome is unknown but is associated with the inflammation within the eyes and may be autoimmune.</t>
+        </is>
+      </c>
+      <c r="L203" s="4" t="inlineStr">
+        <is>
+          <t>Iaconetta 2005; https://pubmed.ncbi.nlm.nih.gov/16109058/</t>
+        </is>
+      </c>
       <c r="M203" s="2" t="inlineStr">
         <is>
-          <t>Systemic</t>
-        </is>
-      </c>
-      <c r="N203" s="2" t="inlineStr"/>
-      <c r="O203" s="2" t="inlineStr"/>
+          <t>Nervous System</t>
+        </is>
+      </c>
+      <c r="N203" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
+      <c r="O203" s="2" t="inlineStr">
+        <is>
+          <t>Unconfirmed</t>
+        </is>
+      </c>
       <c r="P203" s="2" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001203</t>
+          <t>ARI:0001204</t>
         </is>
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001203</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001204</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Tolosa-Hunt syndrome</t>
+          <t>Transverse myelitis</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
         <is>
-          <t>Non-specific inflammation of the cavernous sinus; Non-specific inflammation of the superior orbital fissure; Painful Ophthalmoplegia; THS</t>
+          <t>Secondary acute transverse myelitis</t>
         </is>
       </c>
       <c r="E204" s="4" t="inlineStr"/>
       <c r="F204" s="3" t="inlineStr">
         <is>
-          <t>95794005</t>
+          <t>16631009</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr"/>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>4317989</t>
+          <t>443904</t>
         </is>
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>95794005</t>
+          <t>16631009</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr"/>
       <c r="K204" s="4" t="inlineStr">
         <is>
-          <t>Patients with Tolosa-Hunt syndrome experience episodes of severe headaches surrounding the eyes, along with restricted eye movement that is painful (ophthalmoplegia). Normally, only one eye is affected and will frequently appear protruded. Symptoms may also include nerve abnormalities, such as eyelid drooping, double vision, large pupil, and numbness of the face. This disorder typically occurs in relapsing flares. The cause of Tolosa-Hunt syndrome is unknown but is associated with the inflammation within the eyes and may be autoimmune.</t>
+          <t>Inflammation of the spinal cord with neurological effects that go in a transverse (horizontal or bandlike) manner across the body, as opposed to going up or down the spinal cord.</t>
         </is>
       </c>
       <c r="L204" s="4" t="inlineStr">
         <is>
-          <t>Iaconetta 2005; https://pubmed.ncbi.nlm.nih.gov/16109058/</t>
+          <t>Holroyd 2018; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC6078000/</t>
         </is>
       </c>
       <c r="M204" s="2" t="inlineStr">
         <is>
-          <t>Nervous System</t>
+          <t>Musculoskeletal</t>
         </is>
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Antibody</t>
         </is>
       </c>
       <c r="O204" s="2" t="inlineStr">
         <is>
-          <t>Unconfirmed</t>
+          <t>Autoimmune</t>
         </is>
       </c>
       <c r="P204" s="2" t="n">
@@ -13540,60 +13556,57 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001204</t>
+          <t>ARI:0001205</t>
         </is>
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001204</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001205</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Transverse myelitis</t>
-        </is>
-      </c>
-      <c r="D205" s="4" t="inlineStr">
-        <is>
-          <t>Secondary acute transverse myelitis</t>
-        </is>
-      </c>
+          <t>Ulcerative colitis</t>
+        </is>
+      </c>
+      <c r="D205" s="4" t="inlineStr"/>
       <c r="E205" s="4" t="inlineStr"/>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>16631009</t>
+          <t>64766004</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr"/>
       <c r="H205" s="3" t="inlineStr">
         <is>
-          <t>443904</t>
+          <t>81893</t>
         </is>
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>16631009</t>
+          <t>64766004</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr"/>
       <c r="K205" s="4" t="inlineStr">
         <is>
-          <t>Inflammation of the spinal cord with neurological effects that go in a transverse (horizontal or bandlike) manner across the body, as opposed to going up or down the spinal cord.</t>
+          <t>Ulcerative colitis (UC) is an inflammatory bowel disease (IBD) that causes long-lasting inflammation and sores, called ulcers, in the large intestine, including the colon.  When the condition affects the entire digestive tract, it is called Crohn's disease (CD).
+Both UC and CD are caused by an autoimmune response that reflects the involvement of the innate and adaptive immune systems. The disease mechanism is complex, but appears to start when a normal immune response to a bacterial infection does not stop properly after the infection is fought off. The resulting inflammation leads to the symptoms of both UC and CD.</t>
         </is>
       </c>
       <c r="L205" s="4" t="inlineStr">
         <is>
-          <t>Holroyd 2018; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC6078000/</t>
+          <t>Dahlhamer 2016; https://pubmed.ncbi.nlm.nih.gov/27787492/</t>
         </is>
       </c>
       <c r="M205" s="2" t="inlineStr">
         <is>
-          <t>Musculoskeletal</t>
+          <t>Digestive system</t>
         </is>
       </c>
       <c r="N205" s="2" t="inlineStr">
         <is>
-          <t>Antibody</t>
+          <t>Immune-mediated</t>
         </is>
       </c>
       <c r="O205" s="2" t="inlineStr">
@@ -13608,62 +13621,65 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001205</t>
+          <t>ARI:0001206</t>
         </is>
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001205</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001206</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Ulcerative colitis</t>
-        </is>
-      </c>
-      <c r="D206" s="4" t="inlineStr"/>
+          <t>Undifferentiated connective tissue disease</t>
+        </is>
+      </c>
+      <c r="D206" s="4" t="inlineStr">
+        <is>
+          <t>UCTD; Undifferentiated connective tissue syndrome</t>
+        </is>
+      </c>
       <c r="E206" s="4" t="inlineStr"/>
       <c r="F206" s="3" t="inlineStr">
         <is>
-          <t>64766004</t>
+          <t>239918008</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr"/>
       <c r="H206" s="3" t="inlineStr">
         <is>
-          <t>81893</t>
+          <t>4344165</t>
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>64766004</t>
+          <t>239918008</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr"/>
       <c r="K206" s="4" t="inlineStr">
         <is>
-          <t>Ulcerative colitis (UC) is an inflammatory bowel disease (IBD) that causes long-lasting inflammation and sores, called ulcers, in the large intestine, including the colon.  When the condition affects the entire digestive tract, it is called Crohn's disease (CD).
-Both UC and CD are caused by an autoimmune response that reflects the involvement of the innate and adaptive immune systems. The disease mechanism is complex, but appears to start when a normal immune response to a bacterial infection does not stop properly after the infection is fought off. The resulting inflammation leads to the symptoms of both UC and CD.</t>
+          <t xml:space="preserve">Patients of undifferentiated connective tissue disease (UCTD) share some, but not all, symptoms with other connective tissue diseases, such as systemic lupus erythmatosus, systemic sclerosis, dermatomyositis, polymyositis, rheumatoid arthritis, Sjogren's syndrome, and antiphospholipid syndrome.  UCTD is diagnosed when a patient has a positive serum ANA test and shows stable symptoms for a minimum of 3 years.  UCTD is distinct from the other above-mentioned diseases in that the condition remains stable over time without worsening. 30% of patients diagnosed with UCTD will be given a new diagnosis because their disease will not remain stable.  </t>
         </is>
       </c>
       <c r="L206" s="4" t="inlineStr">
         <is>
-          <t>Dahlhamer 2016; https://pubmed.ncbi.nlm.nih.gov/27787492/</t>
+          <t>Spinillo 2017; https://pubmed.ncbi.nlm.nih.gov/28921728/</t>
         </is>
       </c>
       <c r="M206" s="2" t="inlineStr">
         <is>
-          <t>Digestive system</t>
+          <t>Systemic</t>
         </is>
       </c>
       <c r="N206" s="2" t="inlineStr">
         <is>
-          <t>Immune-mediated</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="O206" s="2" t="inlineStr">
         <is>
-          <t>Autoimmune</t>
+          <t>Unconfirmed</t>
         </is>
       </c>
       <c r="P206" s="2" t="n">
@@ -13673,126 +13689,131 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001206</t>
+          <t>ARI:0001207</t>
         </is>
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001206</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001207</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Undifferentiated connective tissue disease</t>
-        </is>
-      </c>
-      <c r="D207" s="4" t="inlineStr">
-        <is>
-          <t>UCTD; Undifferentiated connective tissue syndrome</t>
-        </is>
-      </c>
+          <t>Urticarial vasculitis</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr"/>
       <c r="E207" s="4" t="inlineStr"/>
       <c r="F207" s="3" t="inlineStr">
         <is>
-          <t>239918008</t>
+          <t>402656007</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr"/>
       <c r="H207" s="3" t="inlineStr">
         <is>
-          <t>4344165</t>
+          <t>4292532</t>
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>239918008</t>
+          <t>402656007</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr"/>
       <c r="K207" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Patients of undifferentiated connective tissue disease (UCTD) share some, but not all, symptoms with other connective tissue diseases, such as systemic lupus erythmatosus, systemic sclerosis, dermatomyositis, polymyositis, rheumatoid arthritis, Sjogren's syndrome, and antiphospholipid syndrome.  UCTD is diagnosed when a patient has a positive serum ANA test and shows stable symptoms for a minimum of 3 years.  UCTD is distinct from the other above-mentioned diseases in that the condition remains stable over time without worsening. 30% of patients diagnosed with UCTD will be given a new diagnosis because their disease will not remain stable.  </t>
-        </is>
-      </c>
-      <c r="L207" s="4" t="inlineStr">
-        <is>
-          <t>Spinillo 2017; https://pubmed.ncbi.nlm.nih.gov/28921728/</t>
-        </is>
-      </c>
-      <c r="M207" s="2" t="inlineStr">
-        <is>
-          <t>Systemic</t>
-        </is>
-      </c>
-      <c r="N207" s="2" t="inlineStr">
-        <is>
-          <t>Unconfirmed</t>
-        </is>
-      </c>
-      <c r="O207" s="2" t="inlineStr">
-        <is>
-          <t>Unconfirmed</t>
-        </is>
-      </c>
-      <c r="P207" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001207</t>
-        </is>
-      </c>
-      <c r="B208" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001207</t>
-        </is>
-      </c>
-      <c r="C208" s="2" t="inlineStr">
-        <is>
-          <t>Urticarial vasculitis</t>
-        </is>
-      </c>
-      <c r="D208" s="4" t="inlineStr"/>
-      <c r="E208" s="4" t="inlineStr"/>
-      <c r="F208" s="3" t="inlineStr">
-        <is>
-          <t>402656007</t>
-        </is>
-      </c>
-      <c r="G208" s="2" t="inlineStr"/>
-      <c r="H208" s="3" t="inlineStr">
-        <is>
-          <t>4292532</t>
-        </is>
-      </c>
-      <c r="I208" s="2" t="inlineStr">
-        <is>
-          <t>402656007</t>
-        </is>
-      </c>
-      <c r="J208" s="2" t="inlineStr"/>
-      <c r="K208" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Autoimmune urticaria occurs when the immune system attacks the normal tissues of the body, resulting in hives. The condition becomes chronic when the lesions persists longer than 6 weeks. Chronic autoimmune urticaria has been found to be associated with autoimmune thyroid disease.
 Urticaria can also be caused by allergic reaction to plants like poison ivy, dyes found in clothing, and cosmetics. An allergic reaction is not an autoimmune disease because there is no involvement by the adaptive immune system and auto-antibodies that attack your own cells are not involved. There are antibodies (IgE antibodies), but they target the invading molecules (e.g., poison ivy), not the cells in the skin. In autoimmune urticaria, the antibodies created are attacking the skin itself, not an invading molecule. 
 </t>
         </is>
       </c>
+      <c r="L207" s="4" t="inlineStr">
+        <is>
+          <t>Kolkhir 2020; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC7063238/</t>
+        </is>
+      </c>
+      <c r="M207" s="2" t="inlineStr">
+        <is>
+          <t>Vascular system</t>
+        </is>
+      </c>
+      <c r="N207" s="2" t="inlineStr">
+        <is>
+          <t>Antibody</t>
+        </is>
+      </c>
+      <c r="O207" s="2" t="inlineStr">
+        <is>
+          <t>Autoimmune</t>
+        </is>
+      </c>
+      <c r="P207" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>ARI:0001208</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001208</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>Uveitis</t>
+        </is>
+      </c>
+      <c r="D208" s="4" t="inlineStr">
+        <is>
+          <t>Autoimmune uveitis; Idiopathic uveitis; Idiopathic intermediate uveitis</t>
+        </is>
+      </c>
+      <c r="E208" s="4" t="inlineStr">
+        <is>
+          <t>Idiopathic Anterior Uveitis</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>128473001, 231947004</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr"/>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>4028363, 4335981</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>128473001, 231947004</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr"/>
+      <c r="K208" s="4" t="inlineStr">
+        <is>
+          <t>Uveitis is an inflammation of the uvea - a set of tissues that form a layer of eyeball that sits between the outer layers of the eye and the "vitreous chamber", which forms the main body of the eye. The uvea itself has several kinds of tissue that can be affected by immune processes, all of which are called uveitis. About half of people who receive a diagnosis of uveitis have an autoimmune form of the disease. Uveitis is a term that means "inflammation of the uvea", and not all forms of uveitis are autoimmune, and not all individuals diagnosed with uveitis have an autoimmune form of uveitis. 
+The most common form of autoimmune uveitis is &lt;a href="&lt;a href="https://diseases.autoimmuneregistry.org/Disease_Profile/intermediate-uveitis"&gt;intermediate uveitis&lt;/a&gt;.</t>
+        </is>
+      </c>
       <c r="L208" s="4" t="inlineStr">
         <is>
-          <t>Kolkhir 2020; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC7063238/</t>
+          <t>Acharya 2013; https://pubmed.ncbi.nlm.nih.gov/24008391/</t>
         </is>
       </c>
       <c r="M208" s="2" t="inlineStr">
         <is>
-          <t>Vascular system</t>
+          <t>Eye</t>
         </is>
       </c>
       <c r="N208" s="2" t="inlineStr">
         <is>
-          <t>Antibody</t>
+          <t>TCELL</t>
         </is>
       </c>
       <c r="O208" s="2" t="inlineStr">
@@ -13801,71 +13822,67 @@
         </is>
       </c>
       <c r="P208" s="2" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001208</t>
+          <t>ARI:0001209</t>
         </is>
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001208</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001209</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Uveitis</t>
+          <t>Vitiligo</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
         <is>
-          <t>Autoimmune uveitis; Idiopathic uveitis; Idiopathic intermediate uveitis</t>
-        </is>
-      </c>
-      <c r="E209" s="4" t="inlineStr">
-        <is>
-          <t>Idiopathic Anterior Uveitis</t>
-        </is>
-      </c>
+          <t>Leukoderma</t>
+        </is>
+      </c>
+      <c r="E209" s="4" t="inlineStr"/>
       <c r="F209" s="3" t="inlineStr">
         <is>
-          <t>128473001, 231947004</t>
+          <t>56727007</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr"/>
       <c r="H209" s="3" t="inlineStr">
         <is>
-          <t>4028363, 4335981</t>
+          <t>138502</t>
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>128473001, 231947004</t>
+          <t>56727007</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr"/>
       <c r="K209" s="4" t="inlineStr">
         <is>
-          <t>Uveitis is an inflammation of the uvea - a set of tissues that form a layer of eyeball that sits between the outer layers of the eye and the "vitreous chamber", which forms the main body of the eye. The uvea itself has several kinds of tissue that can be affected by immune processes, all of which are called uveitis. About half of people who receive a diagnosis of uveitis have an autoimmune form of the disease. Uveitis is a term that means "inflammation of the uvea", and not all forms of uveitis are autoimmune, and not all individuals diagnosed with uveitis have an autoimmune form of uveitis. 
-The most common form of autoimmune uveitis is &lt;a href="&lt;a href="https://diseases.autoimmuneregistry.org/Disease_Profile/intermediate-uveitis"&gt;intermediate uveitis&lt;/a&gt;.</t>
+          <t>Vitiligo is a disease that causes the loss of skin color in blotches. The extent and rate of color loss from vitiligo is unpredictable. It can affect the skin on any part of your body. It may also affect hair, the inside of the mouth, and even the eyes.
+Normally, the color of hair, skin, and eyes is determined by melanin. Vitiligo occurs when the cells that produce melanin die or stop functioning.</t>
         </is>
       </c>
       <c r="L209" s="4" t="inlineStr">
         <is>
-          <t>Acharya 2013; https://pubmed.ncbi.nlm.nih.gov/24008391/</t>
+          <t>Zhang 2016; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC5038943/</t>
         </is>
       </c>
       <c r="M209" s="2" t="inlineStr">
         <is>
-          <t>Eye</t>
+          <t>Skin</t>
         </is>
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>TCELL</t>
+          <t>Antibody</t>
         </is>
       </c>
       <c r="O209" s="2" t="inlineStr">
@@ -13874,62 +13891,57 @@
         </is>
       </c>
       <c r="P209" s="2" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001209</t>
+          <t>ARI:0001210</t>
         </is>
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001209</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001210</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Vitiligo</t>
-        </is>
-      </c>
-      <c r="D210" s="4" t="inlineStr">
-        <is>
-          <t>Leukoderma</t>
-        </is>
-      </c>
+          <t>Vogt-Koyanagi-Harada disease</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr"/>
       <c r="E210" s="4" t="inlineStr"/>
       <c r="F210" s="3" t="inlineStr">
         <is>
-          <t>56727007</t>
+          <t>193497004</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr"/>
       <c r="H210" s="3" t="inlineStr">
         <is>
-          <t>138502</t>
+          <t>4108968</t>
         </is>
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>56727007</t>
+          <t>193497004</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr"/>
       <c r="K210" s="4" t="inlineStr">
         <is>
-          <t>Vitiligo is a disease that causes the loss of skin color in blotches. The extent and rate of color loss from vitiligo is unpredictable. It can affect the skin on any part of your body. It may also affect hair, the inside of the mouth, and even the eyes.
-Normally, the color of hair, skin, and eyes is determined by melanin. Vitiligo occurs when the cells that produce melanin die or stop functioning.</t>
+          <t>Vogt-Koyanagi-Harada (VKH), is a rare disease that affects multiple systems including the nervous system and skin. The disease results in rapid vision loss as well as loss of hearing and hair. Although the cause of VKH is unknown, researchers believe that it is an immune response to a genetic defect of the Human Leukocyte antigen (HLA). Other researchers believe that there may be a genetic predisposition for VKH and may only be expressed by an environmental trigger.</t>
         </is>
       </c>
       <c r="L210" s="4" t="inlineStr">
         <is>
-          <t>Zhang 2016; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC5038943/</t>
+          <t>Lavezzo 2016; https://pubmed.ncbi.nlm.nih.gov/27008848/</t>
         </is>
       </c>
       <c r="M210" s="2" t="inlineStr">
         <is>
-          <t>Skin</t>
+          <t>Systemic</t>
         </is>
       </c>
       <c r="N210" s="2" t="inlineStr">
@@ -13943,139 +13955,75 @@
         </is>
       </c>
       <c r="P210" s="2" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>ARI:0001210</t>
+          <t>ARI:0001211</t>
         </is>
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001210</t>
+          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001211</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Vogt-Koyanagi-Harada disease</t>
-        </is>
-      </c>
-      <c r="D211" s="4" t="inlineStr"/>
+          <t>Warm autoimmune hemolytic anemia</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>Acquired autoimmune hemolytic anemia; Idiopathic autoimmune hemolytic anemia; Immune hemolytic anemia; Immunohemolytic anemia</t>
+        </is>
+      </c>
       <c r="E211" s="4" t="inlineStr"/>
       <c r="F211" s="3" t="inlineStr">
         <is>
-          <t>193497004</t>
+          <t>3978000</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr"/>
       <c r="H211" s="3" t="inlineStr">
         <is>
-          <t>4108968</t>
+          <t>4219853</t>
         </is>
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>193497004</t>
+          <t>3978000</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr"/>
       <c r="K211" s="4" t="inlineStr">
         <is>
-          <t>Vogt-Koyanagi-Harada (VKH), is a rare disease that affects multiple systems including the nervous system and skin. The disease results in rapid vision loss as well as loss of hearing and hair. Although the cause of VKH is unknown, researchers believe that it is an immune response to a genetic defect of the Human Leukocyte antigen (HLA). Other researchers believe that there may be a genetic predisposition for VKH and may only be expressed by an environmental trigger.</t>
-        </is>
-      </c>
-      <c r="L211" s="4" t="inlineStr">
-        <is>
-          <t>Lavezzo 2016; https://pubmed.ncbi.nlm.nih.gov/27008848/</t>
-        </is>
-      </c>
-      <c r="M211" s="2" t="inlineStr">
-        <is>
-          <t>Systemic</t>
-        </is>
-      </c>
-      <c r="N211" s="2" t="inlineStr">
-        <is>
-          <t>Antibody</t>
-        </is>
-      </c>
-      <c r="O211" s="2" t="inlineStr">
-        <is>
-          <t>Autoimmune</t>
-        </is>
-      </c>
-      <c r="P211" s="2" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" s="2" t="inlineStr">
-        <is>
-          <t>ARI:0001211</t>
-        </is>
-      </c>
-      <c r="B212" s="3" t="inlineStr">
-        <is>
-          <t>https://diseases.autoimmuneregistry.org/disease/ARI_0001211</t>
-        </is>
-      </c>
-      <c r="C212" s="2" t="inlineStr">
-        <is>
-          <t>Warm autoimmune hemolytic anemia</t>
-        </is>
-      </c>
-      <c r="D212" s="4" t="inlineStr">
-        <is>
-          <t>Acquired autoimmune hemolytic anemia; Idiopathic autoimmune hemolytic anemia; Immune hemolytic anemia; Immunohemolytic anemia</t>
-        </is>
-      </c>
-      <c r="E212" s="4" t="inlineStr"/>
-      <c r="F212" s="3" t="inlineStr">
-        <is>
-          <t>3978000</t>
-        </is>
-      </c>
-      <c r="G212" s="2" t="inlineStr"/>
-      <c r="H212" s="3" t="inlineStr">
-        <is>
-          <t>4219853</t>
-        </is>
-      </c>
-      <c r="I212" s="2" t="inlineStr">
-        <is>
-          <t>3978000</t>
-        </is>
-      </c>
-      <c r="J212" s="2" t="inlineStr"/>
-      <c r="K212" s="4" t="inlineStr">
-        <is>
           <t xml:space="preserve">Warm autoimmune hemolytic anemia is caused when a person's antibodies attack and destroy their red blood cells.  Unlike &lt;a href="/Disease_Profile/cold-agglutinin-disease.aspx"&gt;cold agglutinin disease&lt;/a&gt;, the autoimmune destruction of cells occurs when a person's body temperature is normal or above normal.  It leads to low red blood cell levels in the body.  
 Some cases of this disease are caused by medications and are not autoimmune.  </t>
         </is>
       </c>
-      <c r="L212" s="4" t="inlineStr">
+      <c r="L211" s="4" t="inlineStr">
         <is>
           <t>Eaton 2011; https://www.ncbi.nlm.nih.gov/pmc/articles/PMC2892249/</t>
         </is>
       </c>
-      <c r="M212" s="2" t="inlineStr">
+      <c r="M211" s="2" t="inlineStr">
         <is>
           <t>Blood</t>
         </is>
       </c>
-      <c r="N212" s="2" t="inlineStr">
+      <c r="N211" s="2" t="inlineStr">
         <is>
           <t>Antibody</t>
         </is>
       </c>
-      <c r="O212" s="2" t="inlineStr">
+      <c r="O211" s="2" t="inlineStr">
         <is>
           <t>Autoimmune</t>
         </is>
       </c>
-      <c r="P212" s="2" t="n">
+      <c r="P211" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -14660,9 +14608,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId576"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H201" r:id="rId577"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B202" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H202" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B203" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B203" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H203" r:id="rId581"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B204" r:id="rId582"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId583"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H204" r:id="rId584"/>
@@ -14687,9 +14635,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B211" r:id="rId603"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F211" r:id="rId604"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H211" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B212" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H212" r:id="rId608"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>